<commit_message>
Unrecognized revenue comparatives: previous week from last week's deck (7,168 MMAD)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -640,22 +640,34 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>collections_basis</t>
+          <t>ur_prev_source</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>AR paid lines by payment date, amount invoiced (same basis as 'Invoices paid' in the BU meeting report)</t>
+          <t>last week's deck</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>collections_basis</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>AR paid lines by payment date, amount invoiced (same basis as 'Invoices paid' in the BU meeting report)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>deposited_month</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B17" s="4" t="n">
         <v>144.0273779292046</v>
       </c>
     </row>
@@ -15505,7 +15517,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unrecognized suppliers by status, MMAD incl. markup; prev_week_total = previous BU update (incl. markup).</t>
+          <t>Unrecognized suppliers by status, MMAD incl. markup; prev_week_total = last week's deck.</t>
         </is>
       </c>
     </row>
@@ -15681,7 +15693,7 @@
         <v>132.49449971306</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>58.541424083405</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5">
@@ -15779,7 +15791,7 @@
         <v>58.2708675006</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>95.15545376</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
@@ -15828,7 +15840,7 @@
         <v>361.6759480747407</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>113.572382579</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8">
@@ -15877,7 +15889,7 @@
         <v>1381.669342470875</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1539.001549975228</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="9">
@@ -15926,7 +15938,7 @@
         <v>160.25160094989</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>347.1237891044</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10">
@@ -15975,7 +15987,7 @@
         <v>252.212123642212</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>438.1603746820252</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11">
@@ -16024,7 +16036,7 @@
         <v>3270.625336294613</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>3466.546150650921</v>
+        <v>3269</v>
       </c>
     </row>
     <row r="12">
@@ -16073,7 +16085,7 @@
         <v>1511.12911517327</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1735.797329236808</v>
+        <v>1513</v>
       </c>
     </row>
   </sheetData>
@@ -18533,7 +18545,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Total AR stands at 12,397 MMAD (−292 WoW, −456 vs month start). Adding 7,128 MMAD of unrecognized revenue (−666 vs the previous BU update), gross exposure is 19,525 MMAD. Unbilled is 9,479 MMAD (76% of AR, −35 WoW); unpaid is 2,370 MMAD (−258 WoW, −252 vs baseline).</t>
+          <t>Total AR stands at 12,397 MMAD (−292 WoW, −456 vs month start). Adding 7,128 MMAD of unrecognized revenue (−40 vs last week), gross exposure is 19,525 MMAD. Unbilled is 9,479 MMAD (76% of AR, −35 WoW); unpaid is 2,370 MMAD (−258 WoW, −252 vs baseline).</t>
         </is>
       </c>
     </row>
@@ -27078,7 +27090,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>7793.898454071787</v>
+        <v>7168</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>7128.328833819261</v>
@@ -27094,7 +27106,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>20482.87511211708</v>
+        <v>19856.97665804529</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>19525.04076045451</v>
@@ -28224,7 +28236,7 @@
       </c>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="4" t="n">
-        <v>58.541424083405</v>
+        <v>127</v>
       </c>
       <c r="E44" s="4" t="n">
         <v>132.49449971306</v>
@@ -28262,7 +28274,7 @@
       </c>
       <c r="C46" s="3" t="n"/>
       <c r="D46" s="4" t="n">
-        <v>95.15545376</v>
+        <v>58</v>
       </c>
       <c r="E46" s="4" t="n">
         <v>58.2708675006</v>
@@ -28281,7 +28293,7 @@
       </c>
       <c r="C47" s="3" t="n"/>
       <c r="D47" s="4" t="n">
-        <v>113.572382579</v>
+        <v>362</v>
       </c>
       <c r="E47" s="4" t="n">
         <v>361.6759480747407</v>
@@ -28300,7 +28312,7 @@
       </c>
       <c r="C48" s="3" t="n"/>
       <c r="D48" s="4" t="n">
-        <v>1539.001549975228</v>
+        <v>1384</v>
       </c>
       <c r="E48" s="4" t="n">
         <v>1381.669342470875</v>
@@ -28319,7 +28331,7 @@
       </c>
       <c r="C49" s="3" t="n"/>
       <c r="D49" s="4" t="n">
-        <v>347.1237891044</v>
+        <v>203</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>160.25160094989</v>
@@ -28338,7 +28350,7 @@
       </c>
       <c r="C50" s="3" t="n"/>
       <c r="D50" s="4" t="n">
-        <v>438.1603746820252</v>
+        <v>252</v>
       </c>
       <c r="E50" s="4" t="n">
         <v>252.212123642212</v>
@@ -28357,7 +28369,7 @@
       </c>
       <c r="C51" s="3" t="n"/>
       <c r="D51" s="4" t="n">
-        <v>3466.546150650921</v>
+        <v>3269</v>
       </c>
       <c r="E51" s="4" t="n">
         <v>3270.625336294613</v>
@@ -28376,7 +28388,7 @@
       </c>
       <c r="C52" s="3" t="n"/>
       <c r="D52" s="4" t="n">
-        <v>1735.797329236808</v>
+        <v>1513</v>
       </c>
       <c r="E52" s="4" t="n">
         <v>1511.12911517327</v>

</xml_diff>

<commit_message>
Weekly deck: non-OCP and JESA-responsibility slides, DSO, month-start unrecognized reference
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -21,18 +21,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNRECOGNIZED" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UR_ATTACHMENT_STATUS" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UR_PO_SUMMARY" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NONOCP_BU" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NONOCP_PROJECTS" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JESA_UNBILLED_BU" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JESA_UNBILLED_STATUS" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DSO" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15494,7 +15499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -15512,6 +15517,7 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15597,6 +15603,11 @@
           <t>prev_week_total</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>month_start_total</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -15646,6 +15657,9 @@
       <c r="O3" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="P3" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -15695,6 +15709,9 @@
       <c r="O4" s="4" t="n">
         <v>127</v>
       </c>
+      <c r="P4" s="4" t="n">
+        <v>127</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -15744,6 +15761,9 @@
       <c r="O5" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -15793,6 +15813,9 @@
       <c r="O6" s="4" t="n">
         <v>58</v>
       </c>
+      <c r="P6" s="4" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -15842,6 +15865,9 @@
       <c r="O7" s="4" t="n">
         <v>362</v>
       </c>
+      <c r="P7" s="4" t="n">
+        <v>364</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -15891,6 +15917,9 @@
       <c r="O8" s="4" t="n">
         <v>1384</v>
       </c>
+      <c r="P8" s="4" t="n">
+        <v>1385</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -15940,6 +15969,9 @@
       <c r="O9" s="4" t="n">
         <v>203</v>
       </c>
+      <c r="P9" s="4" t="n">
+        <v>225</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -15989,6 +16021,9 @@
       <c r="O10" s="4" t="n">
         <v>252</v>
       </c>
+      <c r="P10" s="4" t="n">
+        <v>252</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -16038,6 +16073,9 @@
       <c r="O11" s="4" t="n">
         <v>3269</v>
       </c>
+      <c r="P11" s="4" t="n">
+        <v>3585</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -16086,6 +16124,9 @@
       </c>
       <c r="O12" s="4" t="n">
         <v>1513</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>1556</v>
       </c>
     </row>
   </sheetData>
@@ -16841,6 +16882,2751 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Non-OCP clients (Client 1 = NON OCP): unbilled and unpaid by BU (MMAD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>month_start</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>prev_week</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>2.26201797</v>
+      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="4" t="n">
+        <v>2.26201797</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>4.264925126666665</v>
+      </c>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="4" t="n">
+        <v>4.264925126666665</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>4.514176030000002</v>
+      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="4" t="n">
+        <v>3.611248320000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>6.08784973</v>
+      </c>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="4" t="n">
+        <v>1.29788225</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0.2612669400000001</v>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="4" t="n">
+        <v>5.40000000037253e-07</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.0653166</v>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="4" t="n">
+        <v>0.326583</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1.1582486911064</v>
+      </c>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="4" t="n">
+        <v>0.6521069011064</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>3.1264161761136</v>
+      </c>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="4" t="n">
+        <v>4.92241669044256</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>120.6592861287001</v>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="4" t="n">
+        <v>120.6592861287001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>86.49414509707999</v>
+      </c>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="4" t="n">
+        <v>80.65410298910201</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>3.111915560000015</v>
+      </c>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="4" t="n">
+        <v>2.636780870000015</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>9.594969640476386</v>
+      </c>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="4" t="n">
+        <v>10.87328150047639</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>2.172496425315001</v>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="4" t="n">
+        <v>1.086762579015001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>15.72952923527</v>
+      </c>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="4" t="n">
+        <v>12.35789933434</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0.3537536555</v>
+      </c>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="4" t="n">
+        <v>0.3537536555</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>5.5828837618</v>
+      </c>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="4" t="n">
+        <v>5.5828837618</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Non-OCP projects driving unbilled and unpaid (top 40 by total, MMAD, current week).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>wbs</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>unbilled</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Saudi Arabian Mining Company</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>QC.01661.S01</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Ma'aden - Phase 1 of Phosphate 3 complex - EPCM</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>78.37753682789007</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>29.10148833664001</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>C-4.a Pending client PM approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Saudi Arabian Mining Company</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>QC.01921.S02</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 of the Phosphate 3 Complex - Ma'aden</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>33.38811670475008</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>46.61956574277</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Ltd</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>QC.01756.S02</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>L&amp;T Proprietary Equipment &amp; License Fee for PAP, DAP Plants</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>4.71492093</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>MCA - SENEGAL II</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>QC.00929.S01</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>MCA SENEGAL II POWER PMC ROLE</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>4.4162749</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>BNEDT</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>QC.00964.S01</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Université San Pedro AMO</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.0959416</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>4.269464087143051</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Saudi Arabian Mining Company</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>QC.01921.S03</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 of the Phosphate 3 Complex - Ma'aden</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>4.10738528606</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>C-4.a Pending client PM approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>SNIM</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>QC.02270.S02</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>SNIM TO Wave 4</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>4.0836353398</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Jordan Turkiye Fertilizer Company (JTFC)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>QC.01970.S02</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>JTFC DH PAP TDP and PP Testing - License Fee</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>3.437818</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>SNIM</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>QC.01902.S02</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>SNIM MODERNISATION GUELB 1</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>3.37527739</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>COBCO SA</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>QC.01856.S02</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>AZUR PMC ROLE</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>3.05972119</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>C-4.a Pending client PM approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Saudi Arabian Mining Company</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>QC.02293.S02</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>MAADEN CAPITAL GROWTH</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>2.905920992</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Nutrien</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>QC.01238.S07</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Nutrien 2026 Core Washing</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>2.70697518</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Ma'aden</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>QC.01661.S03.L</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Ma’aden Phosphate 3 Project Phase 1 Engineering and Technical Services.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>1.71855854655</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.5582339403000001</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Ministére interieur</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>QC.02276.S01</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Etude technique et suivi de l'installation de rayonnages</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0.62529132</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>1.643578</v>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>CHEMETICS INC</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>QC.00202.S01</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>DETACHEMENT VANCOUVER</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.551102570000001</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>1.29788225</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>WORLEY ARABIA LIMITED</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>QC.02330.S01</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>MAADEN Phos 3 Phase 1_Jesa Profit</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1.763818917692</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>CBG</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>QC.01771.S01</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>ETUDES NORD COGON FEL1 &amp; FEL2 QT230701.1</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1.51386914</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>SNIM</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>QC.02360.S01</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Cadrage SAP S4H SNIM</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>1.499248422</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Saudi Arabian Mining Company</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>QC.02293.S01</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Maaden Capital Growth</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>1.40100494</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>KCH CASABLANCA</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>QC.02259.S01</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>King's college hospital</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1.216512</v>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>AGENCE URBAINE DE RABAT-SALE</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>QC.00913.S01</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>ETUDE D'ELABORATION DE LA CARTE D'APTITU</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>1.19932</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>OPCI CDG Premium Immo</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>QC.02361.S01</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Aménagement des immeubles Dalil CDG</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0.32992003</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.781224</v>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>ONEE- BRANCHE EAU</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>QC.01235.S02</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Caractérisation des émissions ONEE MOHA</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0.7487892199999999</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.32972</v>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>COBCO SA</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>QC.01793.S01</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>AZUR PROJECT-ESIA STUDY</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>RGS</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>QC.02297.S01</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>RGS - Mission AMO PROJECT</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0.3022103611056</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.5061417904425599</v>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>TARIK OUALALOU ARCHITECTE</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>QC.01142.S01</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Etude d'Aménagement du littoral du Grand</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>DIRECTION DES AMENAGEMENTS HYDRAULIQUES</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>QC.02307.S01</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Etude &amp;Suivi Trvx barrages Rehamna</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0.67716648</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Office de la Formation Professionne</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>QC.01261.S01</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>OFPPT BTP Multiple Tracks Training Prog</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.18134163</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.4861742833333331</v>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Fox River</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>QC.00923.S06</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Fox River Variability Testing</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0.6519670964999998</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Ma'aden</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>QC.01661.S02.O</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Ma’aden Phosphate 3 Project Phase 1 Engineering and Technical Services.</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.37144601436</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.2082063369</v>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>J-7.a Under investigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>DIRECTION DES AMENAGEMENTS HYDRAULIQUES</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>QC.02316.S01</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>ETUDE ET SUIVI DES BARRAGES ESSAOUIRA</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.5443954</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Ideal Development for Manufacturing Industries (IDMI)</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>QC.01247.S04</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>2604-JT-P1810 IDMI Bene Plant Audit</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.43799496</v>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>SGTM</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>QC.01088.S01</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>ETUDE BARRAGE SANGUIN</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.39255187</v>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Ma'aden</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>QC.01661.S02.L</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Ma’aden Phosphate 3 Project Phase 1 Engineering and Technical Services.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.241813130625</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.14535977187</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>BANQUE CENTRALE POPULAIRE</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>QC.00100.S01</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>BCP TOWER</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.359448230000014</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Zenata commercial mall</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>QC.02269.S01</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Zenata mall</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0.35265464</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>MCM-MARINE CONSTRUCTION MAROC</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>QC.01513.S01</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>EXE ACCES PORT DAKHLA</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>0.06000028000000003</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>C-7.a Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Ma'aden</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>QC.01661.S03.E</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Ma’aden Phosphate 3 Project Phase 1 Engineering and Technical Services.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0.32690358459</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>J-2.a Pending JESA PM approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>SNIM</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>QC.02174.S02</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Due Diligence on ElAouj Iron Ore Project</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0.2913869105</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>FNX-INNOV INC</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>QC.01226.S01</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Etude d'Assainissement de la ville Rosso</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.2847</v>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>C-7.b Past due</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unbilled where the action sits with JESA (J-* statuses except SS postponed), by BU and PSR (labor) / Procurement (non-labor), MMAD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>month_start</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>prev_week</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>43.88841028008387</v>
+      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="4" t="n">
+        <v>34.40179050008392</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>153.0893177671223</v>
+      </c>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="4" t="n">
+        <v>137.8581264031223</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>74.85880802481653</v>
+      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="4" t="n">
+        <v>52.59092250481653</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>214.5546040094988</v>
+      </c>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="4" t="n">
+        <v>166.1324606794988</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>19.93161590999955</v>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="4" t="n">
+        <v>17.62053646999955</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>347.3680594096</v>
+      </c>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="4" t="n">
+        <v>285.56024437</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>22.61758495264055</v>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="4" t="n">
+        <v>18.12105508064053</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>-56.61318959164977</v>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="4" t="n">
+        <v>-86.53937665164989</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>11.36061419110639</v>
+      </c>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="4" t="n">
+        <v>6.395188861106397</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1.546770704200003</v>
+      </c>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="4" t="n">
+        <v>1.546770704200003</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>46.66674829190013</v>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="4" t="n">
+        <v>45.02706064190011</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>-12.8384088285</v>
+      </c>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="4" t="n">
+        <v>-12.8384088285</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>35.33577778000013</v>
+      </c>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="4" t="n">
+        <v>34.96368752000013</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>1.346440600000001</v>
+      </c>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="4" t="n">
+        <v>1.295115400000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>4.069733395081001</v>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="4" t="n">
+        <v>3.573264689567001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>-1.186415686175001</v>
+      </c>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="4" t="n">
+        <v>-1.186415686175001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>20.41556775550001</v>
+      </c>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="4" t="n">
+        <v>13.6966085955</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>2.04183504</v>
+      </c>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="4" t="n">
+        <v>2.04183504</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unbilled under JESA responsibility by status and PSR / Procurement (MMAD, current week).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>labor</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>non_labor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>J-3.a Signed by client, pending JESA SS submission</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>21.27779666570502</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>251.6710676252</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>89.75289489471614</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>103.9799279148</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>J-1.e Under JESA PC review</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>3.523243781173918</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>79.37015611472673</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>J-7.a Under investigation</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>14.28215213703128</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>62.46919847820032</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>J-1.d Under JESA finance review</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>14.33829798669951</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>39.67259445221897</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>J-5.a Rejected by client</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>2.63140419</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>46.82484310000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>J-1.c Pending LS milestone</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>43.91690488461226</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>J-4.a Ongoing invoicing</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>12.81371310799999</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>20.12923447000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>J-1.b Pending attachments JESA PA</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2.708838790000004</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>4.39250438</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>J-1.f Pending LC by PC</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0.9512636973060021</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0.8356632759999959</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>J-2.a Pending JESA PM approval</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>22.23543976836997</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>-117.5166734206499</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DSO excluding advances (days), from the BU meeting Power BI report. Update monthly; 'JESA Group' row = group DSO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>dso_current</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>dso_prior_month</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>JESA Group</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>285</v>
+      </c>
+      <c r="C3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>331</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>376</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>294</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>252</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>462</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>192</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>323</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>317</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Auto-drafted from the numbers; rewrite the wording as needed (max 5 messages).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>body</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total AR down 292 MMAD vs last week and down 456 MMAD vs the month-start (07 Oct) baseline</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Total AR stands at 12,397 MMAD (−292 WoW, −456 vs month start). Adding 7,128 MMAD of unrecognized revenue (−40 vs last week), gross exposure is 19,525 MMAD. Unbilled is 9,479 MMAD (76% of AR, −35 WoW); unpaid is 2,370 MMAD (−258 WoW, −252 vs baseline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Collections: 241 MMAD received in October to date (+24 WoW), 8,082 MMAD YTD</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Invoices paid moved from 217 to 241 MMAD this month (payment date basis, amount invoiced). YTD payments received reach 8,082 MMAD (8.08 Bn MAD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Procurement cash position: net −171 MMAD Jul–Oct including October commitments</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative procurement cash IN of 2,104 MMAD vs cash OUT of 2,276 MMAD (Jul–Sep actuals, Oct actuals to 15/10, plus 321 MMAD of approved and pending October commitments). October alone: 151 MMAD in vs 220 MMAD paid, 321 MMAD still to pay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Payables: 2,144 MMAD of supplier invoices in AP (4411 + parked + downpayments), 1,415 MMAD past due</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2,803 open supplier lines. Parked invoices and 4411 open items dominate; see the AP slide for due-date buckets, tiers and top suppliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Letters of credit: 912 MMAD outstanding on opened LCs, 1,583 MMAD including LCs still to be opened</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>October LC maturities of 156 MMAD are counted as approved payments in the cash position. 675 MMAD falls in 2026 and 908 MMAD in 2027 per the maturity schedule.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -17188,7 +19974,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17387,7 +20173,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17754,7 +20540,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18179,7 +20965,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18496,125 +21282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="120" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Auto-drafted from the numbers; rewrite the wording as needed (max 5 messages).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>body</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Total AR down 292 MMAD vs last week and down 456 MMAD vs the month-start (07 Oct) baseline</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Total AR stands at 12,397 MMAD (−292 WoW, −456 vs month start). Adding 7,128 MMAD of unrecognized revenue (−40 vs last week), gross exposure is 19,525 MMAD. Unbilled is 9,479 MMAD (76% of AR, −35 WoW); unpaid is 2,370 MMAD (−258 WoW, −252 vs baseline).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Collections: 241 MMAD received in October to date (+24 WoW), 8,082 MMAD YTD</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Invoices paid moved from 217 to 241 MMAD this month (payment date basis, amount invoiced). YTD payments received reach 8,082 MMAD (8.08 Bn MAD).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Procurement cash position: net −171 MMAD Jul–Oct including October commitments</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Cumulative procurement cash IN of 2,104 MMAD vs cash OUT of 2,276 MMAD (Jul–Sep actuals, Oct actuals to 15/10, plus 321 MMAD of approved and pending October commitments). October alone: 151 MMAD in vs 220 MMAD paid, 321 MMAD still to pay.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Payables: 2,144 MMAD of supplier invoices in AP (4411 + parked + downpayments), 1,415 MMAD past due</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>2,803 open supplier lines. Parked invoices and 4411 open items dominate; see the AP slide for due-date buckets, tiers and top suppliers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Letters of credit: 912 MMAD outstanding on opened LCs, 1,583 MMAD including LCs still to be opened</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>October LC maturities of 156 MMAD are counted as approved payments in the cash position. 675 MMAD falls in 2026 and 908 MMAD in 2027 per the maturity schedule.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18873,7 +21541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19262,7 +21930,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19470,7 +22138,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19933,7 +22601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20070,7 +22738,232 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key figures (MMAD): AR from the raw AR extract (dashboard rules), unrecognized from the UR consolidation, AP from the supplier invoice file, LC from the bank LC situation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>month_start</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>prev_week</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Advance Payment</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>547.4616826512201</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>547.70852735122</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>548.0215817440002</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>9683.62880464431</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>9513.792499159648</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>9479.103423610219</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>2621.817790321611</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>2627.475631534421</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2369.58692128103</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Total AR</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>12852.90827761714</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>12688.97665804529</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>12396.71192663525</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Unrecognized Revenue (incl. markup)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>7552</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>7168</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>7128.328833819261</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Total NEW AR</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>20404.90827761714</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>19856.97665804529</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>19525.04076045451</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AP Downpayment</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>294.098113889038</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>297.372438494094</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>AP Parked Invoices</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>907.9543131556851</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1036.197180581258</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>AP Invoices 4411</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>848.1844034725473</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>810.0038324700001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>LC</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>914.4175485225716</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>911.8422979867036</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Total Payables incl. LC</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>2964.654379039842</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>3055.415749532056</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20338,7 +23231,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26972,231 +29865,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Key figures (MMAD): AR from the raw AR extract (dashboard rules), unrecognized from the UR consolidation, AP from the supplier invoice file, LC from the bank LC situation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>metric</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>month_start</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>prev_week</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>current</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Advance Payment</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>547.4616826512201</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>547.70852735122</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>548.0215817440002</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Unbilled</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>9683.62880464431</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>9513.792499159648</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>9479.103423610219</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>2621.817790321611</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>2627.475631534421</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>2369.58692128103</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Total AR</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>12852.90827761714</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>12688.97665804529</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>12396.71192663525</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Unrecognized Revenue (incl. markup)</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>7168</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>7128.328833819261</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Total NEW AR</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>19856.97665804529</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>19525.04076045451</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>AP Downpayment</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>294.098113889038</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>297.372438494094</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>AP Parked Invoices</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>907.9543131556851</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>1036.197180581258</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>AP Invoices 4411</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>848.1844034725473</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>810.0038324700001</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>LC</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>914.4175485225716</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>911.8422979867036</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Total Payables incl. LC</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>2964.654379039842</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>3055.415749532056</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -28215,7 +30883,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C43" s="3" t="n"/>
+      <c r="C43" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D43" s="4" t="n">
         <v>0</v>
       </c>
@@ -28234,7 +30904,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C44" s="3" t="n"/>
+      <c r="C44" s="4" t="n">
+        <v>127</v>
+      </c>
       <c r="D44" s="4" t="n">
         <v>127</v>
       </c>
@@ -28253,7 +30925,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C45" s="3" t="n"/>
+      <c r="C45" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D45" s="4" t="n">
         <v>0</v>
       </c>
@@ -28272,7 +30946,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C46" s="3" t="n"/>
+      <c r="C46" s="4" t="n">
+        <v>58</v>
+      </c>
       <c r="D46" s="4" t="n">
         <v>58</v>
       </c>
@@ -28291,7 +30967,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C47" s="3" t="n"/>
+      <c r="C47" s="4" t="n">
+        <v>364</v>
+      </c>
       <c r="D47" s="4" t="n">
         <v>362</v>
       </c>
@@ -28310,7 +30988,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C48" s="3" t="n"/>
+      <c r="C48" s="4" t="n">
+        <v>1385</v>
+      </c>
       <c r="D48" s="4" t="n">
         <v>1384</v>
       </c>
@@ -28329,7 +31009,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C49" s="3" t="n"/>
+      <c r="C49" s="4" t="n">
+        <v>225</v>
+      </c>
       <c r="D49" s="4" t="n">
         <v>203</v>
       </c>
@@ -28348,7 +31030,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C50" s="3" t="n"/>
+      <c r="C50" s="4" t="n">
+        <v>252</v>
+      </c>
       <c r="D50" s="4" t="n">
         <v>252</v>
       </c>
@@ -28367,7 +31051,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C51" s="3" t="n"/>
+      <c r="C51" s="4" t="n">
+        <v>3585</v>
+      </c>
       <c r="D51" s="4" t="n">
         <v>3269</v>
       </c>
@@ -28386,7 +31072,9 @@
           <t>Unrecognized</t>
         </is>
       </c>
-      <c r="C52" s="3" t="n"/>
+      <c r="C52" s="4" t="n">
+        <v>1556</v>
+      </c>
       <c r="D52" s="4" t="n">
         <v>1513</v>
       </c>

</xml_diff>

<commit_message>
Weekly deck: title cards with week-on-week deltas, concise key messages with cash position after approved and pending payments
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -19547,12 +19547,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Total AR down 292 MMAD vs last week and down 456 MMAD vs the month-start (07 Oct) baseline</t>
+          <t>Total AR 12,397 MMAD: −292 vs 14 Oct, −456 vs 07 Oct</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Total AR stands at 12,397 MMAD (−292 WoW, −456 vs month start). Adding 7,128 MMAD of unrecognized revenue (−40 vs last week), gross exposure is 19,525 MMAD. Unbilled is 9,479 MMAD (76% of AR, −35 WoW); unpaid is 2,370 MMAD (−258 WoW, −252 vs baseline).</t>
+          <t>Unbilled 9,479 (−35 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unrecognized revenue 7,128 (−40 WoW, −424 vs 07 Oct); gross exposure 19,525 MMAD (−332 WoW).</t>
         </is>
       </c>
     </row>
@@ -19562,12 +19562,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Collections: 241 MMAD received in October to date (+24 WoW), 8,082 MMAD YTD</t>
+          <t>Invoices paid in October to 20 Oct: 241 MMAD (+24 vs 14 Oct); 8,082 MMAD year to date</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Invoices paid moved from 217 to 241 MMAD this month (payment date basis, amount invoiced). YTD payments received reach 8,082 MMAD (8.08 Bn MAD).</t>
+          <t>Invoices deposited in October: 144 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19577,12 +19577,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Procurement cash position: net −171 MMAD Jul–Oct including October commitments</t>
+          <t>Procurement cash Jul–Oct: +150 MMAD on actuals, −107 after approved payments, −171 after pending payments</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Cumulative procurement cash IN of 2,104 MMAD vs cash OUT of 2,276 MMAD (Jul–Sep actuals, Oct actuals to 15/10, plus 321 MMAD of approved and pending October commitments). October alone: 151 MMAD in vs 220 MMAD paid, 321 MMAD still to pay.</t>
+          <t>Cash IN 2,104 MMAD vs cash OUT 1,954 MMAD paid to 15/10 gives +150 MMAD. Approved payments of 258 MMAD (incl. 156 of October LC maturities) bring the position to −107 MMAD; pending payments of 64 MMAD bring it to −171 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19592,12 +19592,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Payables: 2,144 MMAD of supplier invoices in AP (4411 + parked + downpayments), 1,415 MMAD past due</t>
+          <t>Supplier payables 2,144 MMAD, of which 1,415 MMAD past due</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2,803 open supplier lines. Parked invoices and 4411 open items dominate; see the AP slide for due-date buckets, tiers and top suppliers.</t>
+          <t>Parked invoices 1,036, 4411 open items 810, downpayments 297 MMAD (2,803 open lines).</t>
         </is>
       </c>
     </row>
@@ -19607,12 +19607,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Letters of credit: 912 MMAD outstanding on opened LCs, 1,583 MMAD including LCs still to be opened</t>
+          <t>Letters of credit 1,583 MMAD: 912 on opened LCs, 671 still to be opened</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>October LC maturities of 156 MMAD are counted as approved payments in the cash position. 675 MMAD falls in 2026 and 908 MMAD in 2027 per the maturity schedule.</t>
+          <t>156 MMAD matures in October; 630 MMAD in 2026 and 953 MMAD in 2027.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly deck: agenda slide, BU zooms moved to the end, key messages in deck order, sources & definitions slide
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -19509,7 +19509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -19520,7 +19520,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Auto-drafted from the numbers; rewrite the wording as needed (max 5 messages).</t>
+          <t>Drafted from the figures in deck order; rewrite the wording as needed (max 6 messages).</t>
         </is>
       </c>
     </row>
@@ -19552,7 +19552,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Unbilled 9,479 (−35 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unrecognized revenue 7,128 (−40 WoW, −424 vs 07 Oct); gross exposure 19,525 MMAD (−332 WoW).</t>
+          <t>Unbilled 9,479 (−35 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unbilled under JESA responsibility 720 MMAD (PSR 228 / Procurement 492); non-OCP receivables 252 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19562,12 +19562,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Invoices paid in October to 20 Oct: 241 MMAD (+24 vs 14 Oct); 8,082 MMAD year to date</t>
+          <t>Unrecognized revenue 7,128 MMAD (−40 WoW, −424 vs 07 Oct); gross exposure 19,525 MMAD (−332 WoW)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Invoices deposited in October: 144 MMAD.</t>
+          <t>Executed supplier and equipment scope not yet booked as AR, including the 6% JESA cost + fee.</t>
         </is>
       </c>
     </row>
@@ -19577,12 +19577,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Procurement cash Jul–Oct: +150 MMAD on actuals, −107 after approved payments, −171 after pending payments</t>
+          <t>Invoices paid in October to 20 Oct: 241 MMAD (+24 vs 14 Oct); 8,082 MMAD year to date</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Cash IN 2,104 MMAD vs cash OUT 1,954 MMAD paid to 15/10 gives +150 MMAD. Approved payments of 258 MMAD (incl. 156 of October LC maturities) bring the position to −107 MMAD; pending payments of 64 MMAD bring it to −171 MMAD.</t>
+          <t>Invoices deposited in October: 144 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19592,12 +19592,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Supplier payables 2,144 MMAD, of which 1,415 MMAD past due</t>
+          <t>Procurement cash Jul–Oct: +150 MMAD on actuals, −107 after approved payments, −171 after pending payments</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Parked invoices 1,036, 4411 open items 810, downpayments 297 MMAD (2,803 open lines).</t>
+          <t>Cash IN 2,104 MMAD vs cash OUT 1,954 MMAD paid to 15/10 gives +150 MMAD. Approved payments of 258 MMAD (incl. 156 of October LC maturities) bring the position to −107 MMAD; pending payments of 64 MMAD bring it to −171 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19607,10 +19607,25 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>Supplier payables 2,144 MMAD, of which 1,415 MMAD past due</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Parked invoices 1,036, 4411 open items 810, downpayments 297 MMAD (2,803 open lines).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>Letters of credit 1,583 MMAD: 912 on opened LCs, 671 still to be opened</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>156 MMAD matures in October; 630 MMAD in 2026 and 953 MMAD in 2027.</t>
         </is>

</xml_diff>

<commit_message>
Unrecognized slide to reference layout; align unbilled rule with AR dashboard
- Slide 10 rebuilt: revenue vs supplier-cost cards (revenue = cost x 1.06),
  revenue by BU coloured per BU with WoW deltas, Table 7 suppliers by status
  at cost (equipment / subcontractors), status definitions, footnotes
- ar_engine: unbilled now also excludes C-3.a (pending DP clearing) lines,
  reproducing the processed AR dashboard exactly (12,395.1 / 9,477.5)
- README rules updated; inputs history refreshed

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F417"/>
+  <dimension ref="A1:F416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7334,13 +7334,13 @@
         </is>
       </c>
       <c r="D275" s="4" t="n">
-        <v>110.3506010000001</v>
+        <v>108.7051785900001</v>
       </c>
       <c r="E275" s="4" t="n">
         <v>108.70517859</v>
       </c>
       <c r="F275" s="4" t="n">
-        <v>110.03816402</v>
+        <v>108.39274161</v>
       </c>
     </row>
     <row r="276">
@@ -7502,15 +7502,15 @@
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>C-3.a Pending DP payment / clearing</t>
+          <t>J-1.b Pending attachments JESA PA</t>
         </is>
       </c>
       <c r="D282" s="4" t="n">
-        <v>1.64542241</v>
+        <v>1.346440600000001</v>
       </c>
       <c r="E282" s="3" t="n"/>
       <c r="F282" s="4" t="n">
-        <v>1.64542241</v>
+        <v>1.346440600000001</v>
       </c>
     </row>
     <row r="283">
@@ -7526,15 +7526,15 @@
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>J-1.b Pending attachments JESA PA</t>
+          <t>C-2.a Waiting OCP VAT exemption</t>
         </is>
       </c>
       <c r="D283" s="4" t="n">
-        <v>1.346440600000001</v>
+        <v>0.6837</v>
       </c>
       <c r="E283" s="3" t="n"/>
       <c r="F283" s="4" t="n">
-        <v>1.346440600000001</v>
+        <v>0.6837</v>
       </c>
     </row>
     <row r="284">
@@ -7550,15 +7550,15 @@
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>C-2.a Waiting OCP VAT exemption</t>
+          <t>C-1.a At risk (new project)</t>
         </is>
       </c>
       <c r="D284" s="4" t="n">
-        <v>0.6837</v>
+        <v>0.425162</v>
       </c>
       <c r="E284" s="3" t="n"/>
       <c r="F284" s="4" t="n">
-        <v>0.6837</v>
+        <v>0.425162</v>
       </c>
     </row>
     <row r="285">
@@ -7574,15 +7574,15 @@
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>C-1.a At risk (new project)</t>
+          <t>J-1.f Pending LC by PC</t>
         </is>
       </c>
       <c r="D285" s="4" t="n">
-        <v>0.425162</v>
+        <v>0.12776724</v>
       </c>
       <c r="E285" s="3" t="n"/>
       <c r="F285" s="4" t="n">
-        <v>0.425162</v>
+        <v>0.12776724</v>
       </c>
     </row>
     <row r="286">
@@ -7598,15 +7598,15 @@
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>J-1.f Pending LC by PC</t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="D286" s="4" t="n">
-        <v>0.12776724</v>
+        <v>-0.01967444999999939</v>
       </c>
       <c r="E286" s="3" t="n"/>
       <c r="F286" s="4" t="n">
-        <v>0.12776724</v>
+        <v>-0.01967444999999939</v>
       </c>
     </row>
     <row r="287">
@@ -7617,20 +7617,20 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>J-2.a Pending JESA PM approval</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D287" s="4" t="n">
-        <v>-0.01967444999999939</v>
+        <v>4.6697478</v>
       </c>
       <c r="E287" s="3" t="n"/>
       <c r="F287" s="4" t="n">
-        <v>-0.01967444999999939</v>
+        <v>11.12884361</v>
       </c>
     </row>
     <row r="288">
@@ -7646,15 +7646,15 @@
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D288" s="4" t="n">
-        <v>4.6697478</v>
+        <v>334.9231839804762</v>
       </c>
       <c r="E288" s="3" t="n"/>
       <c r="F288" s="4" t="n">
-        <v>11.12884361</v>
+        <v>330.868192730476</v>
       </c>
     </row>
     <row r="289">
@@ -7670,15 +7670,15 @@
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D289" s="4" t="n">
-        <v>334.9231839804762</v>
+        <v>0</v>
       </c>
       <c r="E289" s="3" t="n"/>
       <c r="F289" s="4" t="n">
-        <v>330.868192730476</v>
+        <v>0</v>
       </c>
     </row>
     <row r="290">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D290" s="4" t="n">
@@ -7713,20 +7713,20 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D291" s="4" t="n">
-        <v>0</v>
+        <v>0.76433731</v>
       </c>
       <c r="E291" s="3" t="n"/>
       <c r="F291" s="4" t="n">
-        <v>0</v>
+        <v>0.76433731</v>
       </c>
     </row>
     <row r="292">
@@ -7742,15 +7742,15 @@
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D292" s="4" t="n">
-        <v>0.76433731</v>
+        <v>5.548438780000001</v>
       </c>
       <c r="E292" s="3" t="n"/>
       <c r="F292" s="4" t="n">
-        <v>0.76433731</v>
+        <v>0.40186493</v>
       </c>
     </row>
     <row r="293">
@@ -7766,15 +7766,15 @@
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D293" s="4" t="n">
-        <v>5.548438780000001</v>
+        <v>300.6199704200001</v>
       </c>
       <c r="E293" s="3" t="n"/>
       <c r="F293" s="4" t="n">
-        <v>0.40186493</v>
+        <v>302.3196491200001</v>
       </c>
     </row>
     <row r="294">
@@ -7790,15 +7790,15 @@
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D294" s="4" t="n">
-        <v>300.6199704200001</v>
+        <v>13.92578047</v>
       </c>
       <c r="E294" s="3" t="n"/>
       <c r="F294" s="4" t="n">
-        <v>302.3196491200001</v>
+        <v>13.92578047</v>
       </c>
     </row>
     <row r="295">
@@ -7814,15 +7814,15 @@
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D295" s="4" t="n">
-        <v>13.92578047</v>
+        <v>2.98129806</v>
       </c>
       <c r="E295" s="3" t="n"/>
       <c r="F295" s="4" t="n">
-        <v>13.92578047</v>
+        <v>2.98129806</v>
       </c>
     </row>
     <row r="296">
@@ -7838,15 +7838,15 @@
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D296" s="4" t="n">
-        <v>2.98129806</v>
+        <v>0</v>
       </c>
       <c r="E296" s="3" t="n"/>
       <c r="F296" s="4" t="n">
-        <v>2.98129806</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D297" s="4" t="n">
@@ -7886,15 +7886,15 @@
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D298" s="4" t="n">
-        <v>0</v>
+        <v>15.75310674047639</v>
       </c>
       <c r="E298" s="3" t="n"/>
       <c r="F298" s="4" t="n">
-        <v>0</v>
+        <v>21.60410645047638</v>
       </c>
     </row>
     <row r="299">
@@ -7905,20 +7905,20 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D299" s="4" t="n">
-        <v>15.75310674047639</v>
+        <v>15.99425982</v>
       </c>
       <c r="E299" s="3" t="n"/>
       <c r="F299" s="4" t="n">
-        <v>21.60410645047638</v>
+        <v>15.57084436</v>
       </c>
     </row>
     <row r="300">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
@@ -7938,11 +7938,11 @@
         </is>
       </c>
       <c r="D300" s="4" t="n">
-        <v>15.99425982</v>
+        <v>0.8551772200000001</v>
       </c>
       <c r="E300" s="3" t="n"/>
       <c r="F300" s="4" t="n">
-        <v>15.57084436</v>
+        <v>10.95251629</v>
       </c>
     </row>
     <row r="301">
@@ -7953,20 +7953,20 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D301" s="4" t="n">
-        <v>0.8551772200000001</v>
+        <v>7.810026700000002</v>
       </c>
       <c r="E301" s="3" t="n"/>
       <c r="F301" s="4" t="n">
-        <v>10.95251629</v>
+        <v>7.810026700000002</v>
       </c>
     </row>
     <row r="302">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
@@ -7986,11 +7986,11 @@
         </is>
       </c>
       <c r="D302" s="4" t="n">
-        <v>7.810026700000002</v>
+        <v>3.48834062</v>
       </c>
       <c r="E302" s="3" t="n"/>
       <c r="F302" s="4" t="n">
-        <v>7.810026700000002</v>
+        <v>3.48834062</v>
       </c>
     </row>
     <row r="303">
@@ -8001,20 +8001,20 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D303" s="4" t="n">
-        <v>3.48834062</v>
+        <v>19.2584201400001</v>
       </c>
       <c r="E303" s="3" t="n"/>
       <c r="F303" s="4" t="n">
-        <v>3.48834062</v>
+        <v>19.2584201400001</v>
       </c>
     </row>
     <row r="304">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
@@ -8034,11 +8034,11 @@
         </is>
       </c>
       <c r="D304" s="4" t="n">
-        <v>19.7535405900001</v>
+        <v>2.3234858</v>
       </c>
       <c r="E304" s="3" t="n"/>
       <c r="F304" s="4" t="n">
-        <v>19.7535405900001</v>
+        <v>2.14715848</v>
       </c>
     </row>
     <row r="305">
@@ -8049,20 +8049,20 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D305" s="4" t="n">
-        <v>2.3234858</v>
+        <v>13.39325711</v>
       </c>
       <c r="E305" s="3" t="n"/>
       <c r="F305" s="4" t="n">
-        <v>2.14715848</v>
+        <v>13.39325711</v>
       </c>
     </row>
     <row r="306">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
@@ -8082,11 +8082,11 @@
         </is>
       </c>
       <c r="D306" s="4" t="n">
-        <v>14.54355907</v>
+        <v>13.90425678</v>
       </c>
       <c r="E306" s="3" t="n"/>
       <c r="F306" s="4" t="n">
-        <v>14.54355907</v>
+        <v>11.88657808</v>
       </c>
     </row>
     <row r="307">
@@ -8097,20 +8097,20 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D307" s="4" t="n">
-        <v>13.90425678</v>
+        <v>89.3565952</v>
       </c>
       <c r="E307" s="3" t="n"/>
       <c r="F307" s="4" t="n">
-        <v>11.88657808</v>
+        <v>89.04415822</v>
       </c>
     </row>
     <row r="308">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
@@ -8130,11 +8130,11 @@
         </is>
       </c>
       <c r="D308" s="4" t="n">
-        <v>89.3565952</v>
+        <v>318.8453440404761</v>
       </c>
       <c r="E308" s="3" t="n"/>
       <c r="F308" s="4" t="n">
-        <v>89.04415822</v>
+        <v>313.3461155504761</v>
       </c>
     </row>
     <row r="309">
@@ -8145,20 +8145,20 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D309" s="4" t="n">
-        <v>318.8453440404761</v>
+        <v>0</v>
       </c>
       <c r="E309" s="3" t="n"/>
       <c r="F309" s="4" t="n">
-        <v>313.3461155504761</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310">
@@ -8169,7 +8169,7 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
@@ -8178,35 +8178,37 @@
         </is>
       </c>
       <c r="D310" s="4" t="n">
-        <v>0</v>
+        <v>0.17632732</v>
       </c>
       <c r="E310" s="3" t="n"/>
       <c r="F310" s="4" t="n">
-        <v>0</v>
+        <v>0.17632732</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="3" t="inlineStr">
         <is>
-          <t>Building &amp; Infrastructure</t>
+          <t>JESA Technologies</t>
         </is>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="D311" s="4" t="n">
-        <v>0.17632732</v>
-      </c>
-      <c r="E311" s="3" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E311" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F311" s="4" t="n">
-        <v>0.17632732</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312">
@@ -8222,17 +8224,17 @@
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>Under JESA</t>
         </is>
       </c>
       <c r="D312" s="4" t="n">
-        <v>0</v>
+        <v>2.883317708906</v>
       </c>
       <c r="E312" s="4" t="n">
-        <v>0</v>
+        <v>3.264376512791999</v>
       </c>
       <c r="F312" s="4" t="n">
-        <v>0</v>
+        <v>2.386849003392</v>
       </c>
     </row>
     <row r="313">
@@ -8248,17 +8250,17 @@
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Under JESA</t>
+          <t>Under OCP</t>
         </is>
       </c>
       <c r="D313" s="4" t="n">
-        <v>2.883317708906</v>
+        <v>5.481413554157475</v>
       </c>
       <c r="E313" s="4" t="n">
-        <v>3.264376512791999</v>
+        <v>4.892148413371476</v>
       </c>
       <c r="F313" s="4" t="n">
-        <v>2.386849003392</v>
+        <v>4.892148413371475</v>
       </c>
     </row>
     <row r="314">
@@ -8274,17 +8276,17 @@
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Under OCP</t>
+          <t>SS postponed</t>
         </is>
       </c>
       <c r="D314" s="4" t="n">
-        <v>5.481413554157475</v>
+        <v>0</v>
       </c>
       <c r="E314" s="4" t="n">
-        <v>4.892148413371476</v>
+        <v>0</v>
       </c>
       <c r="F314" s="4" t="n">
-        <v>4.892148413371475</v>
+        <v>0</v>
       </c>
     </row>
     <row r="315">
@@ -8295,22 +8297,20 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>SS postponed</t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="D315" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E315" s="4" t="n">
-        <v>0</v>
-      </c>
+        <v>3.781961891725001</v>
+      </c>
+      <c r="E315" s="3" t="n"/>
       <c r="F315" s="4" t="n">
-        <v>0</v>
+        <v>3.428398488370001</v>
       </c>
     </row>
     <row r="316">
@@ -8326,15 +8326,15 @@
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>J-2.a Pending JESA PM approval</t>
+          <t>J-1.c Pending LS milestone</t>
         </is>
       </c>
       <c r="D316" s="4" t="n">
-        <v>3.781961891725001</v>
+        <v>3.168025259612</v>
       </c>
       <c r="E316" s="3" t="n"/>
       <c r="F316" s="4" t="n">
-        <v>3.428398488370001</v>
+        <v>3.168025259612</v>
       </c>
     </row>
     <row r="317">
@@ -8350,15 +8350,15 @@
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>J-1.c Pending LS milestone</t>
+          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
         </is>
       </c>
       <c r="D317" s="4" t="n">
-        <v>3.168025259612</v>
+        <v>1.73560689285</v>
       </c>
       <c r="E317" s="3" t="n"/>
       <c r="F317" s="4" t="n">
-        <v>3.168025259612</v>
+        <v>1.73560689285</v>
       </c>
     </row>
     <row r="318">
@@ -8374,15 +8374,15 @@
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
+          <t>C-4.a Pending client PM approval</t>
         </is>
       </c>
       <c r="D318" s="4" t="n">
-        <v>1.73560689285</v>
+        <v>2.183716152166</v>
       </c>
       <c r="E318" s="3" t="n"/>
       <c r="F318" s="4" t="n">
-        <v>1.73560689285</v>
+        <v>1.59445101138</v>
       </c>
     </row>
     <row r="319">
@@ -8398,15 +8398,15 @@
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>C-4.a Pending client PM approval</t>
+          <t>C-1.c Pending client PO</t>
         </is>
       </c>
       <c r="D319" s="4" t="n">
-        <v>2.183716152166</v>
+        <v>1.562090509141476</v>
       </c>
       <c r="E319" s="3" t="n"/>
       <c r="F319" s="4" t="n">
-        <v>1.59445101138</v>
+        <v>1.562090509141476</v>
       </c>
     </row>
     <row r="320">
@@ -8422,15 +8422,15 @@
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>C-1.c Pending client PO</t>
+          <t>J-1.e Under JESA PC review</t>
         </is>
       </c>
       <c r="D320" s="4" t="n">
-        <v>1.562090509141476</v>
+        <v>1.024048771605</v>
       </c>
       <c r="E320" s="3" t="n"/>
       <c r="F320" s="4" t="n">
-        <v>1.562090509141476</v>
+        <v>1.024048771605</v>
       </c>
     </row>
     <row r="321">
@@ -8446,15 +8446,15 @@
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>J-1.e Under JESA PC review</t>
+          <t>J-3.a Signed by client, pending JESA SS submission</t>
         </is>
       </c>
       <c r="D321" s="4" t="n">
-        <v>1.024048771605</v>
+        <v>0</v>
       </c>
       <c r="E321" s="3" t="n"/>
       <c r="F321" s="4" t="n">
-        <v>1.024048771605</v>
+        <v>0.110151975705</v>
       </c>
     </row>
     <row r="322">
@@ -8470,15 +8470,15 @@
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>J-3.a Signed by client, pending JESA SS submission</t>
+          <t>J-4.a Ongoing invoicing</t>
         </is>
       </c>
       <c r="D322" s="4" t="n">
-        <v>0</v>
+        <v>0.79271298417</v>
       </c>
       <c r="E322" s="3" t="n"/>
       <c r="F322" s="4" t="n">
-        <v>0.110151975705</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323">
@@ -8494,15 +8494,15 @@
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>J-4.a Ongoing invoicing</t>
+          <t>J-7.a Under investigation</t>
         </is>
       </c>
       <c r="D323" s="4" t="n">
-        <v>0.79271298417</v>
+        <v>-0.04680692892600002</v>
       </c>
       <c r="E323" s="3" t="n"/>
       <c r="F323" s="4" t="n">
-        <v>0</v>
+        <v>-0.04680692892600002</v>
       </c>
     </row>
     <row r="324">
@@ -8518,15 +8518,15 @@
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>J-7.a Under investigation</t>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
         </is>
       </c>
       <c r="D324" s="4" t="n">
-        <v>-0.04680692892600002</v>
+        <v>-1.0254600125</v>
       </c>
       <c r="E324" s="3" t="n"/>
       <c r="F324" s="4" t="n">
-        <v>-0.04680692892600002</v>
+        <v>-1.0254600125</v>
       </c>
     </row>
     <row r="325">
@@ -8542,15 +8542,15 @@
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>J-1.a Pending JESA DMR / attachment creation</t>
+          <t>J-1.d Under JESA finance review</t>
         </is>
       </c>
       <c r="D325" s="4" t="n">
-        <v>-1.0254600125</v>
+        <v>-1.163035417780001</v>
       </c>
       <c r="E325" s="3" t="n"/>
       <c r="F325" s="4" t="n">
-        <v>-1.0254600125</v>
+        <v>-1.163035417780001</v>
       </c>
     </row>
     <row r="326">
@@ -8566,15 +8566,15 @@
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>J-1.d Under JESA finance review</t>
+          <t>J-1.f Pending LC by PC</t>
         </is>
       </c>
       <c r="D326" s="4" t="n">
-        <v>-1.163035417780001</v>
+        <v>-3.648128839</v>
       </c>
       <c r="E326" s="3" t="n"/>
       <c r="F326" s="4" t="n">
-        <v>-1.163035417780001</v>
+        <v>-3.108473132693999</v>
       </c>
     </row>
     <row r="327">
@@ -8585,20 +8585,20 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>J-1.f Pending LC by PC</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D327" s="4" t="n">
-        <v>-3.648128839</v>
+        <v>3.007867988115</v>
       </c>
       <c r="E327" s="3" t="n"/>
       <c r="F327" s="4" t="n">
-        <v>-3.108473132693999</v>
+        <v>4.357662997185</v>
       </c>
     </row>
     <row r="328">
@@ -8614,15 +8614,15 @@
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D328" s="4" t="n">
-        <v>3.007867988115</v>
+        <v>98.44430211217099</v>
       </c>
       <c r="E328" s="3" t="n"/>
       <c r="F328" s="4" t="n">
-        <v>4.357662997185</v>
+        <v>93.72287720217099</v>
       </c>
     </row>
     <row r="329">
@@ -8638,15 +8638,15 @@
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D329" s="4" t="n">
-        <v>98.44430211217099</v>
+        <v>1.27293828302</v>
       </c>
       <c r="E329" s="3" t="n"/>
       <c r="F329" s="4" t="n">
-        <v>93.72287720217099</v>
+        <v>1.27293828302</v>
       </c>
     </row>
     <row r="330">
@@ -8662,15 +8662,15 @@
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D330" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>0</v>
       </c>
       <c r="E330" s="3" t="n"/>
       <c r="F330" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>0</v>
       </c>
     </row>
     <row r="331">
@@ -8681,20 +8681,20 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D331" s="4" t="n">
-        <v>0</v>
+        <v>1.27293828302</v>
       </c>
       <c r="E331" s="3" t="n"/>
       <c r="F331" s="4" t="n">
-        <v>0</v>
+        <v>1.27293828302</v>
       </c>
     </row>
     <row r="332">
@@ -8710,15 +8710,15 @@
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D332" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>8.16003607675</v>
       </c>
       <c r="E332" s="3" t="n"/>
       <c r="F332" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>8.552402850196</v>
       </c>
     </row>
     <row r="333">
@@ -8734,15 +8734,15 @@
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D333" s="4" t="n">
-        <v>8.16003607675</v>
+        <v>0</v>
       </c>
       <c r="E333" s="3" t="n"/>
       <c r="F333" s="4" t="n">
-        <v>8.552402850196</v>
+        <v>0</v>
       </c>
     </row>
     <row r="334">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D334" s="4" t="n">
@@ -8782,15 +8782,15 @@
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D335" s="4" t="n">
-        <v>0</v>
+        <v>1.945679055026001</v>
       </c>
       <c r="E335" s="3" t="n"/>
       <c r="F335" s="4" t="n">
-        <v>0</v>
+        <v>5.14405600793</v>
       </c>
     </row>
     <row r="336">
@@ -8806,15 +8806,15 @@
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D336" s="4" t="n">
-        <v>1.945679055026001</v>
+        <v>0</v>
       </c>
       <c r="E336" s="3" t="n"/>
       <c r="F336" s="4" t="n">
-        <v>5.14405600793</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337">
@@ -8830,7 +8830,7 @@
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D337" s="4" t="n">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="E337" s="3" t="n"/>
       <c r="F337" s="4" t="n">
-        <v>0</v>
+        <v>0.1525025928449999</v>
       </c>
     </row>
     <row r="338">
@@ -8854,15 +8854,15 @@
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D338" s="4" t="n">
-        <v>0</v>
+        <v>91.34645496851</v>
       </c>
       <c r="E338" s="3" t="n"/>
       <c r="F338" s="4" t="n">
-        <v>0.1525025928449999</v>
+        <v>84.231578748385</v>
       </c>
     </row>
     <row r="339">
@@ -8873,20 +8873,20 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D339" s="4" t="n">
-        <v>91.34645496851</v>
+        <v>0.15513457059</v>
       </c>
       <c r="E339" s="3" t="n"/>
       <c r="F339" s="4" t="n">
-        <v>84.231578748385</v>
+        <v>-0.01879922664000011</v>
       </c>
     </row>
     <row r="340">
@@ -8897,7 +8897,7 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
@@ -8906,11 +8906,11 @@
         </is>
       </c>
       <c r="D340" s="4" t="n">
-        <v>0.15513457059</v>
+        <v>3.007867988115</v>
       </c>
       <c r="E340" s="3" t="n"/>
       <c r="F340" s="4" t="n">
-        <v>-0.01879922664000011</v>
+        <v>4.357662997185</v>
       </c>
     </row>
     <row r="341">
@@ -8921,20 +8921,20 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D341" s="4" t="n">
-        <v>3.007867988115</v>
+        <v>2.97567452751</v>
       </c>
       <c r="E341" s="3" t="n"/>
       <c r="F341" s="4" t="n">
-        <v>4.357662997185</v>
+        <v>2.97567452751</v>
       </c>
     </row>
     <row r="342">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
@@ -8954,11 +8954,11 @@
         </is>
       </c>
       <c r="D342" s="4" t="n">
-        <v>2.97567452751</v>
+        <v>0.459083251446</v>
       </c>
       <c r="E342" s="3" t="n"/>
       <c r="F342" s="4" t="n">
-        <v>2.97567452751</v>
+        <v>0.459083251446</v>
       </c>
     </row>
     <row r="343">
@@ -8969,20 +8969,20 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D343" s="4" t="n">
-        <v>0.459083251446</v>
+        <v>0.7454335781100001</v>
       </c>
       <c r="E343" s="3" t="n"/>
       <c r="F343" s="4" t="n">
-        <v>0.459083251446</v>
+        <v>0.7454335781100001</v>
       </c>
     </row>
     <row r="344">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
@@ -9002,11 +9002,11 @@
         </is>
       </c>
       <c r="D344" s="4" t="n">
-        <v>0.7454335781100001</v>
+        <v>42.235841664975</v>
       </c>
       <c r="E344" s="3" t="n"/>
       <c r="F344" s="4" t="n">
-        <v>0.7454335781100001</v>
+        <v>42.235841664975</v>
       </c>
     </row>
     <row r="345">
@@ -9017,20 +9017,20 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D345" s="4" t="n">
-        <v>42.235841664975</v>
+        <v>-2.899139346849999</v>
       </c>
       <c r="E345" s="3" t="n"/>
       <c r="F345" s="4" t="n">
-        <v>42.235841664975</v>
+        <v>-3.318994886749999</v>
       </c>
     </row>
     <row r="346">
@@ -9041,7 +9041,7 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
@@ -9050,11 +9050,11 @@
         </is>
       </c>
       <c r="D346" s="4" t="n">
-        <v>-2.899139346849999</v>
+        <v>38.87578928002</v>
       </c>
       <c r="E346" s="3" t="n"/>
       <c r="F346" s="4" t="n">
-        <v>-3.318994886749999</v>
+        <v>34.15436437002</v>
       </c>
     </row>
     <row r="347">
@@ -9065,20 +9065,20 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D347" s="4" t="n">
-        <v>38.87578928002</v>
+        <v>7.387627933703477</v>
       </c>
       <c r="E347" s="3" t="n"/>
       <c r="F347" s="4" t="n">
-        <v>34.15436437002</v>
+        <v>6.895683424533477</v>
       </c>
     </row>
     <row r="348">
@@ -9089,7 +9089,7 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
@@ -9098,11 +9098,11 @@
         </is>
       </c>
       <c r="D348" s="4" t="n">
-        <v>7.387627933703477</v>
+        <v>18.14652619875</v>
       </c>
       <c r="E348" s="3" t="n"/>
       <c r="F348" s="4" t="n">
-        <v>6.895683424533477</v>
+        <v>18.14652619875</v>
       </c>
     </row>
     <row r="349">
@@ -9113,20 +9113,20 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D349" s="4" t="n">
-        <v>18.14652619875</v>
+        <v>0</v>
       </c>
       <c r="E349" s="3" t="n"/>
       <c r="F349" s="4" t="n">
-        <v>18.14652619875</v>
+        <v>0</v>
       </c>
     </row>
     <row r="350">
@@ -9137,7 +9137,7 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
@@ -9156,23 +9156,25 @@
     <row r="351">
       <c r="A351" s="3" t="inlineStr">
         <is>
-          <t>JESA Technologies</t>
+          <t>Advisory</t>
         </is>
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="D351" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E351" s="3" t="n"/>
+      <c r="E351" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F351" s="4" t="n">
         <v>0</v>
       </c>
@@ -9190,17 +9192,17 @@
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>Under JESA</t>
         </is>
       </c>
       <c r="D352" s="4" t="n">
-        <v>0</v>
+        <v>20.41556775550001</v>
       </c>
       <c r="E352" s="4" t="n">
-        <v>0</v>
+        <v>20.0032397555</v>
       </c>
       <c r="F352" s="4" t="n">
-        <v>0</v>
+        <v>13.6966085955</v>
       </c>
     </row>
     <row r="353">
@@ -9216,17 +9218,17 @@
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Under JESA</t>
+          <t>Under OCP</t>
         </is>
       </c>
       <c r="D353" s="4" t="n">
-        <v>20.41556775550001</v>
+        <v>25.11669179</v>
       </c>
       <c r="E353" s="4" t="n">
-        <v>20.0032397555</v>
+        <v>21.58585378999999</v>
       </c>
       <c r="F353" s="4" t="n">
-        <v>13.6966085955</v>
+        <v>27.89248495</v>
       </c>
     </row>
     <row r="354">
@@ -9242,17 +9244,17 @@
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>Under OCP</t>
+          <t>SS postponed</t>
         </is>
       </c>
       <c r="D354" s="4" t="n">
-        <v>25.11669179</v>
+        <v>0</v>
       </c>
       <c r="E354" s="4" t="n">
-        <v>21.58585378999999</v>
+        <v>0</v>
       </c>
       <c r="F354" s="4" t="n">
-        <v>27.89248495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="355">
@@ -9263,22 +9265,20 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>SS postponed</t>
+          <t>C-4.a Pending client PM approval</t>
         </is>
       </c>
       <c r="D355" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E355" s="4" t="n">
-        <v>0</v>
-      </c>
+        <v>10.10989354</v>
+      </c>
+      <c r="E355" s="3" t="n"/>
       <c r="F355" s="4" t="n">
-        <v>0</v>
+        <v>15.30647778</v>
       </c>
     </row>
     <row r="356">
@@ -9294,15 +9294,15 @@
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>C-4.a Pending client PM approval</t>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
         </is>
       </c>
       <c r="D356" s="4" t="n">
-        <v>10.10989354</v>
+        <v>19.82471001050001</v>
       </c>
       <c r="E356" s="3" t="n"/>
       <c r="F356" s="4" t="n">
-        <v>15.30647778</v>
+        <v>12.0219518505</v>
       </c>
     </row>
     <row r="357">
@@ -9318,15 +9318,15 @@
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>J-1.a Pending JESA DMR / attachment creation</t>
+          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
         </is>
       </c>
       <c r="D357" s="4" t="n">
-        <v>19.82471001050001</v>
+        <v>9.438410930000002</v>
       </c>
       <c r="E357" s="3" t="n"/>
       <c r="F357" s="4" t="n">
-        <v>12.0219518505</v>
+        <v>9.034256850000002</v>
       </c>
     </row>
     <row r="358">
@@ -9342,15 +9342,15 @@
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
+          <t>C-1.c Pending client PO</t>
         </is>
       </c>
       <c r="D358" s="4" t="n">
-        <v>9.438410930000002</v>
+        <v>4.072588319999999</v>
       </c>
       <c r="E358" s="3" t="n"/>
       <c r="F358" s="4" t="n">
-        <v>9.034256850000002</v>
+        <v>3.55175032</v>
       </c>
     </row>
     <row r="359">
@@ -9366,15 +9366,15 @@
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>C-1.c Pending client PO</t>
+          <t>J-4.a Ongoing invoicing</t>
         </is>
       </c>
       <c r="D359" s="4" t="n">
-        <v>4.072588319999999</v>
+        <v>0.412</v>
       </c>
       <c r="E359" s="3" t="n"/>
       <c r="F359" s="4" t="n">
-        <v>3.55175032</v>
+        <v>1.495799</v>
       </c>
     </row>
     <row r="360">
@@ -9390,15 +9390,15 @@
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>J-4.a Ongoing invoicing</t>
+          <t>J-7.a Under investigation</t>
         </is>
       </c>
       <c r="D360" s="4" t="n">
-        <v>0.412</v>
+        <v>0.178857745</v>
       </c>
       <c r="E360" s="3" t="n"/>
       <c r="F360" s="4" t="n">
-        <v>1.495799</v>
+        <v>0.178857745</v>
       </c>
     </row>
     <row r="361">
@@ -9414,15 +9414,15 @@
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>J-7.a Under investigation</t>
+          <t>C-6.a Pending SS OCP rejection</t>
         </is>
       </c>
       <c r="D361" s="4" t="n">
-        <v>0.178857745</v>
+        <v>1.495799</v>
       </c>
       <c r="E361" s="3" t="n"/>
       <c r="F361" s="4" t="n">
-        <v>0.178857745</v>
+        <v>0</v>
       </c>
     </row>
     <row r="362">
@@ -9433,20 +9433,20 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>C-6.a Pending SS OCP rejection</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D362" s="4" t="n">
-        <v>1.495799</v>
+        <v>7.620723</v>
       </c>
       <c r="E362" s="3" t="n"/>
       <c r="F362" s="4" t="n">
-        <v>0</v>
+        <v>8.241983000000001</v>
       </c>
     </row>
     <row r="363">
@@ -9462,15 +9462,15 @@
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D363" s="4" t="n">
-        <v>7.620723</v>
+        <v>19.8199807618</v>
       </c>
       <c r="E363" s="3" t="n"/>
       <c r="F363" s="4" t="n">
-        <v>8.241983000000001</v>
+        <v>20.0097067618</v>
       </c>
     </row>
     <row r="364">
@@ -9486,15 +9486,15 @@
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D364" s="4" t="n">
-        <v>19.8199807618</v>
+        <v>0</v>
       </c>
       <c r="E364" s="3" t="n"/>
       <c r="F364" s="4" t="n">
-        <v>20.0097067618</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D365" s="4" t="n">
@@ -9529,20 +9529,20 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D366" s="4" t="n">
-        <v>0</v>
+        <v>5.702727</v>
       </c>
       <c r="E366" s="3" t="n"/>
       <c r="F366" s="4" t="n">
-        <v>0</v>
+        <v>5.702727</v>
       </c>
     </row>
     <row r="367">
@@ -9558,15 +9558,15 @@
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D367" s="4" t="n">
-        <v>5.702727</v>
+        <v>0.266</v>
       </c>
       <c r="E367" s="3" t="n"/>
       <c r="F367" s="4" t="n">
-        <v>5.702727</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="368">
@@ -9582,15 +9582,15 @@
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D368" s="4" t="n">
-        <v>0.266</v>
+        <v>0</v>
       </c>
       <c r="E368" s="3" t="n"/>
       <c r="F368" s="4" t="n">
-        <v>0.266</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D369" s="4" t="n">
@@ -9630,15 +9630,15 @@
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D370" s="4" t="n">
-        <v>0</v>
+        <v>5.599305</v>
       </c>
       <c r="E370" s="3" t="n"/>
       <c r="F370" s="4" t="n">
-        <v>0</v>
+        <v>3.010328</v>
       </c>
     </row>
     <row r="371">
@@ -9654,15 +9654,15 @@
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D371" s="4" t="n">
-        <v>5.599305</v>
+        <v>0</v>
       </c>
       <c r="E371" s="3" t="n"/>
       <c r="F371" s="4" t="n">
-        <v>3.010328</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372">
@@ -9678,7 +9678,7 @@
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D372" s="4" t="n">
@@ -9702,15 +9702,15 @@
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D373" s="4" t="n">
-        <v>0</v>
+        <v>15.8726717618</v>
       </c>
       <c r="E373" s="3" t="n"/>
       <c r="F373" s="4" t="n">
-        <v>0</v>
+        <v>19.2726347618</v>
       </c>
     </row>
     <row r="374">
@@ -9721,20 +9721,20 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D374" s="4" t="n">
-        <v>15.8726717618</v>
+        <v>7.449941010000002</v>
       </c>
       <c r="E374" s="3" t="n"/>
       <c r="F374" s="4" t="n">
-        <v>19.2726347618</v>
+        <v>7.500495880000001</v>
       </c>
     </row>
     <row r="375">
@@ -9745,7 +9745,7 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
@@ -9754,11 +9754,11 @@
         </is>
       </c>
       <c r="D375" s="4" t="n">
-        <v>7.449941010000002</v>
+        <v>1.966475</v>
       </c>
       <c r="E375" s="3" t="n"/>
       <c r="F375" s="4" t="n">
-        <v>7.500495880000001</v>
+        <v>6.410291</v>
       </c>
     </row>
     <row r="376">
@@ -9769,20 +9769,20 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D376" s="4" t="n">
-        <v>1.966475</v>
+        <v>3.019860209999999</v>
       </c>
       <c r="E376" s="3" t="n"/>
       <c r="F376" s="4" t="n">
-        <v>6.410291</v>
+        <v>2.776067639999999</v>
       </c>
     </row>
     <row r="377">
@@ -9793,7 +9793,7 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
@@ -9802,11 +9802,11 @@
         </is>
       </c>
       <c r="D377" s="4" t="n">
-        <v>3.019860209999999</v>
+        <v>3.31</v>
       </c>
       <c r="E377" s="3" t="n"/>
       <c r="F377" s="4" t="n">
-        <v>2.776067639999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="378">
@@ -9817,20 +9817,20 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D378" s="4" t="n">
-        <v>3.31</v>
+        <v>5.90244817</v>
       </c>
       <c r="E378" s="3" t="n"/>
       <c r="F378" s="4" t="n">
-        <v>0</v>
+        <v>5.09577917</v>
       </c>
     </row>
     <row r="379">
@@ -9841,7 +9841,7 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
@@ -9850,11 +9850,11 @@
         </is>
       </c>
       <c r="D379" s="4" t="n">
-        <v>5.90244817</v>
+        <v>3.330940422</v>
       </c>
       <c r="E379" s="3" t="n"/>
       <c r="F379" s="4" t="n">
-        <v>5.09577917</v>
+        <v>3.330940422</v>
       </c>
     </row>
     <row r="380">
@@ -9865,20 +9865,20 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D380" s="4" t="n">
-        <v>3.330940422</v>
+        <v>1.97228386</v>
       </c>
       <c r="E380" s="3" t="n"/>
       <c r="F380" s="4" t="n">
-        <v>3.330940422</v>
+        <v>1.97228386</v>
       </c>
     </row>
     <row r="381">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
@@ -9898,11 +9898,11 @@
         </is>
       </c>
       <c r="D381" s="4" t="n">
-        <v>1.97228386</v>
+        <v>10.3206683398</v>
       </c>
       <c r="E381" s="3" t="n"/>
       <c r="F381" s="4" t="n">
-        <v>1.97228386</v>
+        <v>10.3206683398</v>
       </c>
     </row>
     <row r="382">
@@ -9913,20 +9913,20 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D382" s="4" t="n">
-        <v>10.3206683398</v>
+        <v>27.1877262955</v>
       </c>
       <c r="E382" s="3" t="n"/>
       <c r="F382" s="4" t="n">
-        <v>10.3206683398</v>
+        <v>24.2444669955</v>
       </c>
     </row>
     <row r="383">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
@@ -9946,11 +9946,11 @@
         </is>
       </c>
       <c r="D383" s="4" t="n">
-        <v>27.1877262955</v>
+        <v>8.51262</v>
       </c>
       <c r="E383" s="3" t="n"/>
       <c r="F383" s="4" t="n">
-        <v>24.2444669955</v>
+        <v>8.18979</v>
       </c>
     </row>
     <row r="384">
@@ -9961,20 +9961,20 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D384" s="4" t="n">
-        <v>8.51262</v>
+        <v>0</v>
       </c>
       <c r="E384" s="3" t="n"/>
       <c r="F384" s="4" t="n">
-        <v>8.18979</v>
+        <v>0</v>
       </c>
     </row>
     <row r="385">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
@@ -10004,23 +10004,25 @@
     <row r="386">
       <c r="A386" s="3" t="inlineStr">
         <is>
-          <t>Advisory</t>
+          <t>Building &amp; Capabilities</t>
         </is>
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="D386" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E386" s="3" t="n"/>
+      <c r="E386" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F386" s="4" t="n">
         <v>0</v>
       </c>
@@ -10038,17 +10040,17 @@
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>Under JESA</t>
         </is>
       </c>
       <c r="D387" s="4" t="n">
-        <v>0</v>
+        <v>2.04183504</v>
       </c>
       <c r="E387" s="4" t="n">
-        <v>0</v>
+        <v>2.04183504</v>
       </c>
       <c r="F387" s="4" t="n">
-        <v>0</v>
+        <v>2.04183504</v>
       </c>
     </row>
     <row r="388">
@@ -10064,17 +10066,17 @@
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Under JESA</t>
+          <t>Under OCP</t>
         </is>
       </c>
       <c r="D388" s="4" t="n">
-        <v>2.04183504</v>
+        <v>3.94193829</v>
       </c>
       <c r="E388" s="4" t="n">
-        <v>2.04183504</v>
+        <v>3.941938290000001</v>
       </c>
       <c r="F388" s="4" t="n">
-        <v>2.04183504</v>
+        <v>3.94193829</v>
       </c>
     </row>
     <row r="389">
@@ -10090,17 +10092,17 @@
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>Under OCP</t>
+          <t>SS postponed</t>
         </is>
       </c>
       <c r="D389" s="4" t="n">
-        <v>3.94193829</v>
+        <v>0</v>
       </c>
       <c r="E389" s="4" t="n">
-        <v>3.941938290000001</v>
+        <v>0</v>
       </c>
       <c r="F389" s="4" t="n">
-        <v>3.94193829</v>
+        <v>0</v>
       </c>
     </row>
     <row r="390">
@@ -10111,22 +10113,20 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>SS postponed</t>
+          <t>C-4.a Pending client PM approval</t>
         </is>
       </c>
       <c r="D390" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E390" s="4" t="n">
-        <v>0</v>
-      </c>
+        <v>3.94193829</v>
+      </c>
+      <c r="E390" s="3" t="n"/>
       <c r="F390" s="4" t="n">
-        <v>0</v>
+        <v>3.94193829</v>
       </c>
     </row>
     <row r="391">
@@ -10142,15 +10142,15 @@
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>C-4.a Pending client PM approval</t>
+          <t>J-1.b Pending attachments JESA PA</t>
         </is>
       </c>
       <c r="D391" s="4" t="n">
-        <v>3.94193829</v>
+        <v>1.42969378</v>
       </c>
       <c r="E391" s="3" t="n"/>
       <c r="F391" s="4" t="n">
-        <v>3.94193829</v>
+        <v>1.42969378</v>
       </c>
     </row>
     <row r="392">
@@ -10166,15 +10166,15 @@
       </c>
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>J-1.b Pending attachments JESA PA</t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="D392" s="4" t="n">
-        <v>1.42969378</v>
+        <v>0.61214126</v>
       </c>
       <c r="E392" s="3" t="n"/>
       <c r="F392" s="4" t="n">
-        <v>1.42969378</v>
+        <v>0.61214126</v>
       </c>
     </row>
     <row r="393">
@@ -10185,20 +10185,20 @@
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>J-2.a Pending JESA PM approval</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D393" s="4" t="n">
-        <v>0.61214126</v>
+        <v>0.3396483899999996</v>
       </c>
       <c r="E393" s="3" t="n"/>
       <c r="F393" s="4" t="n">
-        <v>0.61214126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="394">
@@ -10214,15 +10214,15 @@
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D394" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>1.08369285</v>
       </c>
       <c r="E394" s="3" t="n"/>
       <c r="F394" s="4" t="n">
-        <v>0</v>
+        <v>1.42334124</v>
       </c>
     </row>
     <row r="395">
@@ -10238,15 +10238,15 @@
       </c>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D395" s="4" t="n">
-        <v>1.08369285</v>
+        <v>0</v>
       </c>
       <c r="E395" s="3" t="n"/>
       <c r="F395" s="4" t="n">
-        <v>1.42334124</v>
+        <v>0</v>
       </c>
     </row>
     <row r="396">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D396" s="4" t="n">
@@ -10281,12 +10281,12 @@
       </c>
       <c r="B397" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D397" s="4" t="n">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D398" s="4" t="n">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D399" s="4" t="n">
@@ -10358,15 +10358,15 @@
       </c>
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D400" s="4" t="n">
-        <v>0</v>
+        <v>1.08369285</v>
       </c>
       <c r="E400" s="3" t="n"/>
       <c r="F400" s="4" t="n">
-        <v>0</v>
+        <v>1.08369285</v>
       </c>
     </row>
     <row r="401">
@@ -10382,15 +10382,15 @@
       </c>
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D401" s="4" t="n">
-        <v>1.08369285</v>
+        <v>0</v>
       </c>
       <c r="E401" s="3" t="n"/>
       <c r="F401" s="4" t="n">
-        <v>1.08369285</v>
+        <v>0</v>
       </c>
     </row>
     <row r="402">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D402" s="4" t="n">
@@ -10430,7 +10430,7 @@
       </c>
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D403" s="4" t="n">
@@ -10454,15 +10454,15 @@
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D404" s="4" t="n">
-        <v>0</v>
+        <v>0.3396483899999996</v>
       </c>
       <c r="E404" s="3" t="n"/>
       <c r="F404" s="4" t="n">
-        <v>0</v>
+        <v>0.3396483899999996</v>
       </c>
     </row>
     <row r="405">
@@ -10473,20 +10473,20 @@
       </c>
       <c r="B405" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D405" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0.4907168099999997</v>
       </c>
       <c r="E405" s="3" t="n"/>
       <c r="F405" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0.4907168099999997</v>
       </c>
     </row>
     <row r="406">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B406" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C406" s="3" t="inlineStr">
@@ -10506,11 +10506,11 @@
         </is>
       </c>
       <c r="D406" s="4" t="n">
-        <v>0.4907168099999997</v>
+        <v>0</v>
       </c>
       <c r="E406" s="3" t="n"/>
       <c r="F406" s="4" t="n">
-        <v>0.4907168099999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="407">
@@ -10521,20 +10521,20 @@
       </c>
       <c r="B407" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C407" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D407" s="4" t="n">
-        <v>0</v>
+        <v>0.22973683</v>
       </c>
       <c r="E407" s="3" t="n"/>
       <c r="F407" s="4" t="n">
-        <v>0</v>
+        <v>0.22973683</v>
       </c>
     </row>
     <row r="408">
@@ -10545,7 +10545,7 @@
       </c>
       <c r="B408" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C408" s="3" t="inlineStr">
@@ -10554,11 +10554,11 @@
         </is>
       </c>
       <c r="D408" s="4" t="n">
-        <v>0.22973683</v>
+        <v>0.7691738100000001</v>
       </c>
       <c r="E408" s="3" t="n"/>
       <c r="F408" s="4" t="n">
-        <v>0.22973683</v>
+        <v>0.7691738100000001</v>
       </c>
     </row>
     <row r="409">
@@ -10569,20 +10569,20 @@
       </c>
       <c r="B409" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C409" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D409" s="4" t="n">
-        <v>0.7691738100000001</v>
+        <v>0.6202166199999994</v>
       </c>
       <c r="E409" s="3" t="n"/>
       <c r="F409" s="4" t="n">
-        <v>0.7691738100000001</v>
+        <v>0.6202166199999994</v>
       </c>
     </row>
     <row r="410">
@@ -10593,7 +10593,7 @@
       </c>
       <c r="B410" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C410" s="3" t="inlineStr">
@@ -10602,11 +10602,11 @@
         </is>
       </c>
       <c r="D410" s="4" t="n">
-        <v>0.6202166199999994</v>
+        <v>0.31451904</v>
       </c>
       <c r="E410" s="3" t="n"/>
       <c r="F410" s="4" t="n">
-        <v>0.6202166199999994</v>
+        <v>0.31451904</v>
       </c>
     </row>
     <row r="411">
@@ -10617,20 +10617,20 @@
       </c>
       <c r="B411" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D411" s="4" t="n">
-        <v>0.31451904</v>
+        <v>0.8676346699999999</v>
       </c>
       <c r="E411" s="3" t="n"/>
       <c r="F411" s="4" t="n">
-        <v>0.31451904</v>
+        <v>0.8676346699999999</v>
       </c>
     </row>
     <row r="412">
@@ -10641,7 +10641,7 @@
       </c>
       <c r="B412" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C412" s="3" t="inlineStr">
@@ -10650,11 +10650,11 @@
         </is>
       </c>
       <c r="D412" s="4" t="n">
-        <v>0.8676346699999999</v>
+        <v>0</v>
       </c>
       <c r="E412" s="3" t="n"/>
       <c r="F412" s="4" t="n">
-        <v>0.8676346699999999</v>
+        <v>0.3396483899999996</v>
       </c>
     </row>
     <row r="413">
@@ -10665,20 +10665,20 @@
       </c>
       <c r="B413" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D413" s="4" t="n">
-        <v>0</v>
+        <v>3.775468400000001</v>
       </c>
       <c r="E413" s="3" t="n"/>
       <c r="F413" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>3.775468400000001</v>
       </c>
     </row>
     <row r="414">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B414" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C414" s="3" t="inlineStr">
@@ -10698,11 +10698,11 @@
         </is>
       </c>
       <c r="D414" s="4" t="n">
-        <v>3.775468400000001</v>
+        <v>0</v>
       </c>
       <c r="E414" s="3" t="n"/>
       <c r="F414" s="4" t="n">
-        <v>3.775468400000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="415">
@@ -10713,12 +10713,12 @@
       </c>
       <c r="B415" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D415" s="4" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B416" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C416" s="3" t="inlineStr">
@@ -10746,34 +10746,10 @@
         </is>
       </c>
       <c r="D416" s="4" t="n">
-        <v>0</v>
+        <v>0.3396483899999996</v>
       </c>
       <c r="E416" s="3" t="n"/>
       <c r="F416" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="417">
-      <c r="A417" s="3" t="inlineStr">
-        <is>
-          <t>Building &amp; Capabilities</t>
-        </is>
-      </c>
-      <c r="B417" s="3" t="inlineStr">
-        <is>
-          <t>aging_unpaid</t>
-        </is>
-      </c>
-      <c r="C417" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D417" s="4" t="n">
-        <v>0.3396483899999996</v>
-      </c>
-      <c r="E417" s="3" t="n"/>
-      <c r="F417" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -19547,12 +19523,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Total AR 12,397 MMAD: −292 vs 14 Oct, −456 vs 07 Oct</t>
+          <t>Total AR 12,395 MMAD: −294 vs 14 Oct, −456 vs 07 Oct</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Unbilled 9,479 (−35 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unbilled under JESA responsibility 720 MMAD (PSR 228 / Procurement 492); non-OCP receivables 252 MMAD.</t>
+          <t>Unbilled 9,477 (−37 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unbilled under JESA responsibility 720 MMAD (PSR 228 / Procurement 492); non-OCP receivables 252 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19562,7 +19538,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Unrecognized revenue 7,128 MMAD (−40 WoW, −424 vs 07 Oct); gross exposure 19,525 MMAD (−332 WoW)</t>
+          <t>Unrecognized revenue 7,128 MMAD (−40 WoW, −424 vs 07 Oct); gross exposure 19,523 MMAD (−334 WoW)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -22820,13 +22796,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>9683.62880464431</v>
+        <v>9681.98338223431</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>9513.792499159648</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>9479.103423610219</v>
+        <v>9477.458001200219</v>
       </c>
     </row>
     <row r="5">
@@ -22852,13 +22828,13 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>12852.90827761714</v>
+        <v>12851.26285520714</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>12688.97665804529</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>12396.71192663525</v>
+        <v>12395.06650422525</v>
       </c>
     </row>
     <row r="7">
@@ -22884,13 +22860,13 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>20404.90827761714</v>
+        <v>20403.26285520714</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>19856.97665804529</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>19525.04076045451</v>
+        <v>19523.39533804451</v>
       </c>
     </row>
     <row r="9">
@@ -29929,7 +29905,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8108.709021648703</v>
+        <v>8107.063599238703</v>
       </c>
     </row>
     <row r="5">
@@ -29949,7 +29925,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>6222.058062918043</v>
+        <v>6220.412640508043</v>
       </c>
     </row>
     <row r="7">
@@ -29979,7 +29955,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>12145.1699950181</v>
+        <v>12143.5245726081</v>
       </c>
     </row>
     <row r="10">
@@ -30584,13 +30560,13 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>147.4579813800002</v>
+        <v>145.8125589700002</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>145.5530990800001</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>146.7221289400002</v>
+        <v>145.0767065300002</v>
       </c>
     </row>
     <row r="29">
@@ -30626,13 +30602,13 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>487.0509131604763</v>
+        <v>485.4054907504762</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>486.3849952404764</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>488.7191652804763</v>
+        <v>487.0737428704763</v>
       </c>
     </row>
     <row r="31">
@@ -31710,13 +31686,13 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>110.3506010000001</v>
+        <v>108.7051785900001</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>108.70517859</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>110.03816402</v>
+        <v>108.39274161</v>
       </c>
     </row>
     <row r="30">
@@ -32003,7 +31979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -32496,17 +32472,17 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>C-3.a Pending DP payment / clearing</t>
+          <t>C-2.a Waiting OCP VAT exemption</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1.64542241</v>
+        <v>1.50242933</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0</v>
+        <v>1.50242933</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>1.64542241</v>
+        <v>1.50242933</v>
       </c>
     </row>
     <row r="25">
@@ -32517,17 +32493,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>C-2.a Waiting OCP VAT exemption</t>
+          <t>C-1.e Waiting mirror POs for PDR</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1.50242933</v>
+        <v>0.10387899</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>1.50242933</v>
+        <v>0</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>1.50242933</v>
+        <v>0.10387899</v>
       </c>
     </row>
     <row r="26">
@@ -32538,58 +32514,37 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>C-1.e Waiting mirror POs for PDR</t>
+          <t xml:space="preserve">PENDING OCP </t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>0.10387899</v>
+        <v>0</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.10387899</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>OCP</t>
+          <t>JESA</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PENDING OCP </t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0</v>
+        <v>-46.80343063892482</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0</v>
+        <v>-62.59554572227994</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>JESA</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>J-2.a Pending JESA PM approval</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>-46.80343063892482</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>-62.59554572227994</v>
-      </c>
-      <c r="E28" s="4" t="n">
         <v>-95.28123365227995</v>
       </c>
     </row>
@@ -32922,13 +32877,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>8277.110015976186</v>
+        <v>8275.464593566185</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>8120.680624622309</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>8018.910507052301</v>
+        <v>8017.265084642301</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Keep DP-clearing lines in unbilled (BU meeting basis)
- ar_engine: C-3.a lines stay in unbilled; totals back to 12,396.7 / 9,479.1
- README: note the 1.6 MMAD difference vs the processed dashboard
- inputs history refreshed

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F416"/>
+  <dimension ref="A1:F417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7334,13 +7334,13 @@
         </is>
       </c>
       <c r="D275" s="4" t="n">
-        <v>108.7051785900001</v>
+        <v>110.3506010000001</v>
       </c>
       <c r="E275" s="4" t="n">
         <v>108.70517859</v>
       </c>
       <c r="F275" s="4" t="n">
-        <v>108.39274161</v>
+        <v>110.03816402</v>
       </c>
     </row>
     <row r="276">
@@ -7502,15 +7502,15 @@
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>J-1.b Pending attachments JESA PA</t>
+          <t>C-3.a Pending DP payment / clearing</t>
         </is>
       </c>
       <c r="D282" s="4" t="n">
-        <v>1.346440600000001</v>
+        <v>1.64542241</v>
       </c>
       <c r="E282" s="3" t="n"/>
       <c r="F282" s="4" t="n">
-        <v>1.346440600000001</v>
+        <v>1.64542241</v>
       </c>
     </row>
     <row r="283">
@@ -7526,15 +7526,15 @@
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>C-2.a Waiting OCP VAT exemption</t>
+          <t>J-1.b Pending attachments JESA PA</t>
         </is>
       </c>
       <c r="D283" s="4" t="n">
-        <v>0.6837</v>
+        <v>1.346440600000001</v>
       </c>
       <c r="E283" s="3" t="n"/>
       <c r="F283" s="4" t="n">
-        <v>0.6837</v>
+        <v>1.346440600000001</v>
       </c>
     </row>
     <row r="284">
@@ -7550,15 +7550,15 @@
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>C-1.a At risk (new project)</t>
+          <t>C-2.a Waiting OCP VAT exemption</t>
         </is>
       </c>
       <c r="D284" s="4" t="n">
-        <v>0.425162</v>
+        <v>0.6837</v>
       </c>
       <c r="E284" s="3" t="n"/>
       <c r="F284" s="4" t="n">
-        <v>0.425162</v>
+        <v>0.6837</v>
       </c>
     </row>
     <row r="285">
@@ -7574,15 +7574,15 @@
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>J-1.f Pending LC by PC</t>
+          <t>C-1.a At risk (new project)</t>
         </is>
       </c>
       <c r="D285" s="4" t="n">
-        <v>0.12776724</v>
+        <v>0.425162</v>
       </c>
       <c r="E285" s="3" t="n"/>
       <c r="F285" s="4" t="n">
-        <v>0.12776724</v>
+        <v>0.425162</v>
       </c>
     </row>
     <row r="286">
@@ -7598,15 +7598,15 @@
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>J-2.a Pending JESA PM approval</t>
+          <t>J-1.f Pending LC by PC</t>
         </is>
       </c>
       <c r="D286" s="4" t="n">
-        <v>-0.01967444999999939</v>
+        <v>0.12776724</v>
       </c>
       <c r="E286" s="3" t="n"/>
       <c r="F286" s="4" t="n">
-        <v>-0.01967444999999939</v>
+        <v>0.12776724</v>
       </c>
     </row>
     <row r="287">
@@ -7617,20 +7617,20 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="D287" s="4" t="n">
-        <v>4.6697478</v>
+        <v>-0.01967444999999939</v>
       </c>
       <c r="E287" s="3" t="n"/>
       <c r="F287" s="4" t="n">
-        <v>11.12884361</v>
+        <v>-0.01967444999999939</v>
       </c>
     </row>
     <row r="288">
@@ -7646,15 +7646,15 @@
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D288" s="4" t="n">
-        <v>334.9231839804762</v>
+        <v>4.6697478</v>
       </c>
       <c r="E288" s="3" t="n"/>
       <c r="F288" s="4" t="n">
-        <v>330.868192730476</v>
+        <v>11.12884361</v>
       </c>
     </row>
     <row r="289">
@@ -7670,15 +7670,15 @@
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D289" s="4" t="n">
-        <v>0</v>
+        <v>334.9231839804762</v>
       </c>
       <c r="E289" s="3" t="n"/>
       <c r="F289" s="4" t="n">
-        <v>0</v>
+        <v>330.868192730476</v>
       </c>
     </row>
     <row r="290">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D290" s="4" t="n">
@@ -7713,20 +7713,20 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D291" s="4" t="n">
-        <v>0.76433731</v>
+        <v>0</v>
       </c>
       <c r="E291" s="3" t="n"/>
       <c r="F291" s="4" t="n">
-        <v>0.76433731</v>
+        <v>0</v>
       </c>
     </row>
     <row r="292">
@@ -7742,15 +7742,15 @@
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D292" s="4" t="n">
-        <v>5.548438780000001</v>
+        <v>0.76433731</v>
       </c>
       <c r="E292" s="3" t="n"/>
       <c r="F292" s="4" t="n">
-        <v>0.40186493</v>
+        <v>0.76433731</v>
       </c>
     </row>
     <row r="293">
@@ -7766,15 +7766,15 @@
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D293" s="4" t="n">
-        <v>300.6199704200001</v>
+        <v>5.548438780000001</v>
       </c>
       <c r="E293" s="3" t="n"/>
       <c r="F293" s="4" t="n">
-        <v>302.3196491200001</v>
+        <v>0.40186493</v>
       </c>
     </row>
     <row r="294">
@@ -7790,15 +7790,15 @@
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D294" s="4" t="n">
-        <v>13.92578047</v>
+        <v>300.6199704200001</v>
       </c>
       <c r="E294" s="3" t="n"/>
       <c r="F294" s="4" t="n">
-        <v>13.92578047</v>
+        <v>302.3196491200001</v>
       </c>
     </row>
     <row r="295">
@@ -7814,15 +7814,15 @@
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D295" s="4" t="n">
-        <v>2.98129806</v>
+        <v>13.92578047</v>
       </c>
       <c r="E295" s="3" t="n"/>
       <c r="F295" s="4" t="n">
-        <v>2.98129806</v>
+        <v>13.92578047</v>
       </c>
     </row>
     <row r="296">
@@ -7838,15 +7838,15 @@
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D296" s="4" t="n">
-        <v>0</v>
+        <v>2.98129806</v>
       </c>
       <c r="E296" s="3" t="n"/>
       <c r="F296" s="4" t="n">
-        <v>0</v>
+        <v>2.98129806</v>
       </c>
     </row>
     <row r="297">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D297" s="4" t="n">
@@ -7886,15 +7886,15 @@
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D298" s="4" t="n">
-        <v>15.75310674047639</v>
+        <v>0</v>
       </c>
       <c r="E298" s="3" t="n"/>
       <c r="F298" s="4" t="n">
-        <v>21.60410645047638</v>
+        <v>0</v>
       </c>
     </row>
     <row r="299">
@@ -7905,20 +7905,20 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D299" s="4" t="n">
-        <v>15.99425982</v>
+        <v>15.75310674047639</v>
       </c>
       <c r="E299" s="3" t="n"/>
       <c r="F299" s="4" t="n">
-        <v>15.57084436</v>
+        <v>21.60410645047638</v>
       </c>
     </row>
     <row r="300">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
@@ -7938,11 +7938,11 @@
         </is>
       </c>
       <c r="D300" s="4" t="n">
-        <v>0.8551772200000001</v>
+        <v>15.99425982</v>
       </c>
       <c r="E300" s="3" t="n"/>
       <c r="F300" s="4" t="n">
-        <v>10.95251629</v>
+        <v>15.57084436</v>
       </c>
     </row>
     <row r="301">
@@ -7953,20 +7953,20 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D301" s="4" t="n">
-        <v>7.810026700000002</v>
+        <v>0.8551772200000001</v>
       </c>
       <c r="E301" s="3" t="n"/>
       <c r="F301" s="4" t="n">
-        <v>7.810026700000002</v>
+        <v>10.95251629</v>
       </c>
     </row>
     <row r="302">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
@@ -7986,11 +7986,11 @@
         </is>
       </c>
       <c r="D302" s="4" t="n">
-        <v>3.48834062</v>
+        <v>7.810026700000002</v>
       </c>
       <c r="E302" s="3" t="n"/>
       <c r="F302" s="4" t="n">
-        <v>3.48834062</v>
+        <v>7.810026700000002</v>
       </c>
     </row>
     <row r="303">
@@ -8001,20 +8001,20 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D303" s="4" t="n">
-        <v>19.2584201400001</v>
+        <v>3.48834062</v>
       </c>
       <c r="E303" s="3" t="n"/>
       <c r="F303" s="4" t="n">
-        <v>19.2584201400001</v>
+        <v>3.48834062</v>
       </c>
     </row>
     <row r="304">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
@@ -8034,11 +8034,11 @@
         </is>
       </c>
       <c r="D304" s="4" t="n">
-        <v>2.3234858</v>
+        <v>19.7535405900001</v>
       </c>
       <c r="E304" s="3" t="n"/>
       <c r="F304" s="4" t="n">
-        <v>2.14715848</v>
+        <v>19.7535405900001</v>
       </c>
     </row>
     <row r="305">
@@ -8049,20 +8049,20 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D305" s="4" t="n">
-        <v>13.39325711</v>
+        <v>2.3234858</v>
       </c>
       <c r="E305" s="3" t="n"/>
       <c r="F305" s="4" t="n">
-        <v>13.39325711</v>
+        <v>2.14715848</v>
       </c>
     </row>
     <row r="306">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
@@ -8082,11 +8082,11 @@
         </is>
       </c>
       <c r="D306" s="4" t="n">
-        <v>13.90425678</v>
+        <v>14.54355907</v>
       </c>
       <c r="E306" s="3" t="n"/>
       <c r="F306" s="4" t="n">
-        <v>11.88657808</v>
+        <v>14.54355907</v>
       </c>
     </row>
     <row r="307">
@@ -8097,20 +8097,20 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D307" s="4" t="n">
-        <v>89.3565952</v>
+        <v>13.90425678</v>
       </c>
       <c r="E307" s="3" t="n"/>
       <c r="F307" s="4" t="n">
-        <v>89.04415822</v>
+        <v>11.88657808</v>
       </c>
     </row>
     <row r="308">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
@@ -8130,11 +8130,11 @@
         </is>
       </c>
       <c r="D308" s="4" t="n">
-        <v>318.8453440404761</v>
+        <v>89.3565952</v>
       </c>
       <c r="E308" s="3" t="n"/>
       <c r="F308" s="4" t="n">
-        <v>313.3461155504761</v>
+        <v>89.04415822</v>
       </c>
     </row>
     <row r="309">
@@ -8145,20 +8145,20 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D309" s="4" t="n">
-        <v>0</v>
+        <v>318.8453440404761</v>
       </c>
       <c r="E309" s="3" t="n"/>
       <c r="F309" s="4" t="n">
-        <v>0</v>
+        <v>313.3461155504761</v>
       </c>
     </row>
     <row r="310">
@@ -8169,7 +8169,7 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
@@ -8178,37 +8178,35 @@
         </is>
       </c>
       <c r="D310" s="4" t="n">
-        <v>0.17632732</v>
+        <v>0</v>
       </c>
       <c r="E310" s="3" t="n"/>
       <c r="F310" s="4" t="n">
-        <v>0.17632732</v>
+        <v>0</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="3" t="inlineStr">
         <is>
-          <t>JESA Technologies</t>
+          <t>Building &amp; Infrastructure</t>
         </is>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D311" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E311" s="4" t="n">
-        <v>0</v>
-      </c>
+        <v>0.17632732</v>
+      </c>
+      <c r="E311" s="3" t="n"/>
       <c r="F311" s="4" t="n">
-        <v>0</v>
+        <v>0.17632732</v>
       </c>
     </row>
     <row r="312">
@@ -8224,17 +8222,17 @@
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Under JESA</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="D312" s="4" t="n">
-        <v>2.883317708906</v>
+        <v>0</v>
       </c>
       <c r="E312" s="4" t="n">
-        <v>3.264376512791999</v>
+        <v>0</v>
       </c>
       <c r="F312" s="4" t="n">
-        <v>2.386849003392</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313">
@@ -8250,17 +8248,17 @@
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Under OCP</t>
+          <t>Under JESA</t>
         </is>
       </c>
       <c r="D313" s="4" t="n">
-        <v>5.481413554157475</v>
+        <v>2.883317708906</v>
       </c>
       <c r="E313" s="4" t="n">
-        <v>4.892148413371476</v>
+        <v>3.264376512791999</v>
       </c>
       <c r="F313" s="4" t="n">
-        <v>4.892148413371475</v>
+        <v>2.386849003392</v>
       </c>
     </row>
     <row r="314">
@@ -8276,17 +8274,17 @@
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>SS postponed</t>
+          <t>Under OCP</t>
         </is>
       </c>
       <c r="D314" s="4" t="n">
-        <v>0</v>
+        <v>5.481413554157475</v>
       </c>
       <c r="E314" s="4" t="n">
-        <v>0</v>
+        <v>4.892148413371476</v>
       </c>
       <c r="F314" s="4" t="n">
-        <v>0</v>
+        <v>4.892148413371475</v>
       </c>
     </row>
     <row r="315">
@@ -8297,20 +8295,22 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>J-2.a Pending JESA PM approval</t>
+          <t>SS postponed</t>
         </is>
       </c>
       <c r="D315" s="4" t="n">
-        <v>3.781961891725001</v>
-      </c>
-      <c r="E315" s="3" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E315" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F315" s="4" t="n">
-        <v>3.428398488370001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="316">
@@ -8326,15 +8326,15 @@
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>J-1.c Pending LS milestone</t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="D316" s="4" t="n">
-        <v>3.168025259612</v>
+        <v>3.781961891725001</v>
       </c>
       <c r="E316" s="3" t="n"/>
       <c r="F316" s="4" t="n">
-        <v>3.168025259612</v>
+        <v>3.428398488370001</v>
       </c>
     </row>
     <row r="317">
@@ -8350,15 +8350,15 @@
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
+          <t>J-1.c Pending LS milestone</t>
         </is>
       </c>
       <c r="D317" s="4" t="n">
-        <v>1.73560689285</v>
+        <v>3.168025259612</v>
       </c>
       <c r="E317" s="3" t="n"/>
       <c r="F317" s="4" t="n">
-        <v>1.73560689285</v>
+        <v>3.168025259612</v>
       </c>
     </row>
     <row r="318">
@@ -8374,15 +8374,15 @@
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>C-4.a Pending client PM approval</t>
+          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
         </is>
       </c>
       <c r="D318" s="4" t="n">
-        <v>2.183716152166</v>
+        <v>1.73560689285</v>
       </c>
       <c r="E318" s="3" t="n"/>
       <c r="F318" s="4" t="n">
-        <v>1.59445101138</v>
+        <v>1.73560689285</v>
       </c>
     </row>
     <row r="319">
@@ -8398,15 +8398,15 @@
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>C-1.c Pending client PO</t>
+          <t>C-4.a Pending client PM approval</t>
         </is>
       </c>
       <c r="D319" s="4" t="n">
-        <v>1.562090509141476</v>
+        <v>2.183716152166</v>
       </c>
       <c r="E319" s="3" t="n"/>
       <c r="F319" s="4" t="n">
-        <v>1.562090509141476</v>
+        <v>1.59445101138</v>
       </c>
     </row>
     <row r="320">
@@ -8422,15 +8422,15 @@
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>J-1.e Under JESA PC review</t>
+          <t>C-1.c Pending client PO</t>
         </is>
       </c>
       <c r="D320" s="4" t="n">
-        <v>1.024048771605</v>
+        <v>1.562090509141476</v>
       </c>
       <c r="E320" s="3" t="n"/>
       <c r="F320" s="4" t="n">
-        <v>1.024048771605</v>
+        <v>1.562090509141476</v>
       </c>
     </row>
     <row r="321">
@@ -8446,15 +8446,15 @@
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>J-3.a Signed by client, pending JESA SS submission</t>
+          <t>J-1.e Under JESA PC review</t>
         </is>
       </c>
       <c r="D321" s="4" t="n">
-        <v>0</v>
+        <v>1.024048771605</v>
       </c>
       <c r="E321" s="3" t="n"/>
       <c r="F321" s="4" t="n">
-        <v>0.110151975705</v>
+        <v>1.024048771605</v>
       </c>
     </row>
     <row r="322">
@@ -8470,15 +8470,15 @@
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>J-4.a Ongoing invoicing</t>
+          <t>J-3.a Signed by client, pending JESA SS submission</t>
         </is>
       </c>
       <c r="D322" s="4" t="n">
-        <v>0.79271298417</v>
+        <v>0</v>
       </c>
       <c r="E322" s="3" t="n"/>
       <c r="F322" s="4" t="n">
-        <v>0</v>
+        <v>0.110151975705</v>
       </c>
     </row>
     <row r="323">
@@ -8494,15 +8494,15 @@
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>J-7.a Under investigation</t>
+          <t>J-4.a Ongoing invoicing</t>
         </is>
       </c>
       <c r="D323" s="4" t="n">
-        <v>-0.04680692892600002</v>
+        <v>0.79271298417</v>
       </c>
       <c r="E323" s="3" t="n"/>
       <c r="F323" s="4" t="n">
-        <v>-0.04680692892600002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="324">
@@ -8518,15 +8518,15 @@
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>J-1.a Pending JESA DMR / attachment creation</t>
+          <t>J-7.a Under investigation</t>
         </is>
       </c>
       <c r="D324" s="4" t="n">
-        <v>-1.0254600125</v>
+        <v>-0.04680692892600002</v>
       </c>
       <c r="E324" s="3" t="n"/>
       <c r="F324" s="4" t="n">
-        <v>-1.0254600125</v>
+        <v>-0.04680692892600002</v>
       </c>
     </row>
     <row r="325">
@@ -8542,15 +8542,15 @@
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>J-1.d Under JESA finance review</t>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
         </is>
       </c>
       <c r="D325" s="4" t="n">
-        <v>-1.163035417780001</v>
+        <v>-1.0254600125</v>
       </c>
       <c r="E325" s="3" t="n"/>
       <c r="F325" s="4" t="n">
-        <v>-1.163035417780001</v>
+        <v>-1.0254600125</v>
       </c>
     </row>
     <row r="326">
@@ -8566,15 +8566,15 @@
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>J-1.f Pending LC by PC</t>
+          <t>J-1.d Under JESA finance review</t>
         </is>
       </c>
       <c r="D326" s="4" t="n">
-        <v>-3.648128839</v>
+        <v>-1.163035417780001</v>
       </c>
       <c r="E326" s="3" t="n"/>
       <c r="F326" s="4" t="n">
-        <v>-3.108473132693999</v>
+        <v>-1.163035417780001</v>
       </c>
     </row>
     <row r="327">
@@ -8585,20 +8585,20 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>J-1.f Pending LC by PC</t>
         </is>
       </c>
       <c r="D327" s="4" t="n">
-        <v>3.007867988115</v>
+        <v>-3.648128839</v>
       </c>
       <c r="E327" s="3" t="n"/>
       <c r="F327" s="4" t="n">
-        <v>4.357662997185</v>
+        <v>-3.108473132693999</v>
       </c>
     </row>
     <row r="328">
@@ -8614,15 +8614,15 @@
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D328" s="4" t="n">
-        <v>98.44430211217099</v>
+        <v>3.007867988115</v>
       </c>
       <c r="E328" s="3" t="n"/>
       <c r="F328" s="4" t="n">
-        <v>93.72287720217099</v>
+        <v>4.357662997185</v>
       </c>
     </row>
     <row r="329">
@@ -8638,15 +8638,15 @@
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D329" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>98.44430211217099</v>
       </c>
       <c r="E329" s="3" t="n"/>
       <c r="F329" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>93.72287720217099</v>
       </c>
     </row>
     <row r="330">
@@ -8662,15 +8662,15 @@
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D330" s="4" t="n">
-        <v>0</v>
+        <v>1.27293828302</v>
       </c>
       <c r="E330" s="3" t="n"/>
       <c r="F330" s="4" t="n">
-        <v>0</v>
+        <v>1.27293828302</v>
       </c>
     </row>
     <row r="331">
@@ -8681,20 +8681,20 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D331" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>0</v>
       </c>
       <c r="E331" s="3" t="n"/>
       <c r="F331" s="4" t="n">
-        <v>1.27293828302</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332">
@@ -8710,15 +8710,15 @@
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D332" s="4" t="n">
-        <v>8.16003607675</v>
+        <v>1.27293828302</v>
       </c>
       <c r="E332" s="3" t="n"/>
       <c r="F332" s="4" t="n">
-        <v>8.552402850196</v>
+        <v>1.27293828302</v>
       </c>
     </row>
     <row r="333">
@@ -8734,15 +8734,15 @@
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D333" s="4" t="n">
-        <v>0</v>
+        <v>8.16003607675</v>
       </c>
       <c r="E333" s="3" t="n"/>
       <c r="F333" s="4" t="n">
-        <v>0</v>
+        <v>8.552402850196</v>
       </c>
     </row>
     <row r="334">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D334" s="4" t="n">
@@ -8782,15 +8782,15 @@
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D335" s="4" t="n">
-        <v>1.945679055026001</v>
+        <v>0</v>
       </c>
       <c r="E335" s="3" t="n"/>
       <c r="F335" s="4" t="n">
-        <v>5.14405600793</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336">
@@ -8806,15 +8806,15 @@
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D336" s="4" t="n">
-        <v>0</v>
+        <v>1.945679055026001</v>
       </c>
       <c r="E336" s="3" t="n"/>
       <c r="F336" s="4" t="n">
-        <v>0</v>
+        <v>5.14405600793</v>
       </c>
     </row>
     <row r="337">
@@ -8830,7 +8830,7 @@
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D337" s="4" t="n">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="E337" s="3" t="n"/>
       <c r="F337" s="4" t="n">
-        <v>0.1525025928449999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="338">
@@ -8854,15 +8854,15 @@
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D338" s="4" t="n">
-        <v>91.34645496851</v>
+        <v>0</v>
       </c>
       <c r="E338" s="3" t="n"/>
       <c r="F338" s="4" t="n">
-        <v>84.231578748385</v>
+        <v>0.1525025928449999</v>
       </c>
     </row>
     <row r="339">
@@ -8873,20 +8873,20 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D339" s="4" t="n">
-        <v>0.15513457059</v>
+        <v>91.34645496851</v>
       </c>
       <c r="E339" s="3" t="n"/>
       <c r="F339" s="4" t="n">
-        <v>-0.01879922664000011</v>
+        <v>84.231578748385</v>
       </c>
     </row>
     <row r="340">
@@ -8897,7 +8897,7 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
@@ -8906,11 +8906,11 @@
         </is>
       </c>
       <c r="D340" s="4" t="n">
-        <v>3.007867988115</v>
+        <v>0.15513457059</v>
       </c>
       <c r="E340" s="3" t="n"/>
       <c r="F340" s="4" t="n">
-        <v>4.357662997185</v>
+        <v>-0.01879922664000011</v>
       </c>
     </row>
     <row r="341">
@@ -8921,20 +8921,20 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D341" s="4" t="n">
-        <v>2.97567452751</v>
+        <v>3.007867988115</v>
       </c>
       <c r="E341" s="3" t="n"/>
       <c r="F341" s="4" t="n">
-        <v>2.97567452751</v>
+        <v>4.357662997185</v>
       </c>
     </row>
     <row r="342">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
@@ -8954,11 +8954,11 @@
         </is>
       </c>
       <c r="D342" s="4" t="n">
-        <v>0.459083251446</v>
+        <v>2.97567452751</v>
       </c>
       <c r="E342" s="3" t="n"/>
       <c r="F342" s="4" t="n">
-        <v>0.459083251446</v>
+        <v>2.97567452751</v>
       </c>
     </row>
     <row r="343">
@@ -8969,20 +8969,20 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D343" s="4" t="n">
-        <v>0.7454335781100001</v>
+        <v>0.459083251446</v>
       </c>
       <c r="E343" s="3" t="n"/>
       <c r="F343" s="4" t="n">
-        <v>0.7454335781100001</v>
+        <v>0.459083251446</v>
       </c>
     </row>
     <row r="344">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
@@ -9002,11 +9002,11 @@
         </is>
       </c>
       <c r="D344" s="4" t="n">
-        <v>42.235841664975</v>
+        <v>0.7454335781100001</v>
       </c>
       <c r="E344" s="3" t="n"/>
       <c r="F344" s="4" t="n">
-        <v>42.235841664975</v>
+        <v>0.7454335781100001</v>
       </c>
     </row>
     <row r="345">
@@ -9017,20 +9017,20 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D345" s="4" t="n">
-        <v>-2.899139346849999</v>
+        <v>42.235841664975</v>
       </c>
       <c r="E345" s="3" t="n"/>
       <c r="F345" s="4" t="n">
-        <v>-3.318994886749999</v>
+        <v>42.235841664975</v>
       </c>
     </row>
     <row r="346">
@@ -9041,7 +9041,7 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
@@ -9050,11 +9050,11 @@
         </is>
       </c>
       <c r="D346" s="4" t="n">
-        <v>38.87578928002</v>
+        <v>-2.899139346849999</v>
       </c>
       <c r="E346" s="3" t="n"/>
       <c r="F346" s="4" t="n">
-        <v>34.15436437002</v>
+        <v>-3.318994886749999</v>
       </c>
     </row>
     <row r="347">
@@ -9065,20 +9065,20 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D347" s="4" t="n">
-        <v>7.387627933703477</v>
+        <v>38.87578928002</v>
       </c>
       <c r="E347" s="3" t="n"/>
       <c r="F347" s="4" t="n">
-        <v>6.895683424533477</v>
+        <v>34.15436437002</v>
       </c>
     </row>
     <row r="348">
@@ -9089,7 +9089,7 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
@@ -9098,11 +9098,11 @@
         </is>
       </c>
       <c r="D348" s="4" t="n">
-        <v>18.14652619875</v>
+        <v>7.387627933703477</v>
       </c>
       <c r="E348" s="3" t="n"/>
       <c r="F348" s="4" t="n">
-        <v>18.14652619875</v>
+        <v>6.895683424533477</v>
       </c>
     </row>
     <row r="349">
@@ -9113,20 +9113,20 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D349" s="4" t="n">
-        <v>0</v>
+        <v>18.14652619875</v>
       </c>
       <c r="E349" s="3" t="n"/>
       <c r="F349" s="4" t="n">
-        <v>0</v>
+        <v>18.14652619875</v>
       </c>
     </row>
     <row r="350">
@@ -9137,7 +9137,7 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
@@ -9156,25 +9156,23 @@
     <row r="351">
       <c r="A351" s="3" t="inlineStr">
         <is>
-          <t>Advisory</t>
+          <t>JESA Technologies</t>
         </is>
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D351" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E351" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="E351" s="3" t="n"/>
       <c r="F351" s="4" t="n">
         <v>0</v>
       </c>
@@ -9192,17 +9190,17 @@
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Under JESA</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="D352" s="4" t="n">
-        <v>20.41556775550001</v>
+        <v>0</v>
       </c>
       <c r="E352" s="4" t="n">
-        <v>20.0032397555</v>
+        <v>0</v>
       </c>
       <c r="F352" s="4" t="n">
-        <v>13.6966085955</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
@@ -9218,17 +9216,17 @@
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Under OCP</t>
+          <t>Under JESA</t>
         </is>
       </c>
       <c r="D353" s="4" t="n">
-        <v>25.11669179</v>
+        <v>20.41556775550001</v>
       </c>
       <c r="E353" s="4" t="n">
-        <v>21.58585378999999</v>
+        <v>20.0032397555</v>
       </c>
       <c r="F353" s="4" t="n">
-        <v>27.89248495</v>
+        <v>13.6966085955</v>
       </c>
     </row>
     <row r="354">
@@ -9244,17 +9242,17 @@
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>SS postponed</t>
+          <t>Under OCP</t>
         </is>
       </c>
       <c r="D354" s="4" t="n">
-        <v>0</v>
+        <v>25.11669179</v>
       </c>
       <c r="E354" s="4" t="n">
-        <v>0</v>
+        <v>21.58585378999999</v>
       </c>
       <c r="F354" s="4" t="n">
-        <v>0</v>
+        <v>27.89248495</v>
       </c>
     </row>
     <row r="355">
@@ -9265,20 +9263,22 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>C-4.a Pending client PM approval</t>
+          <t>SS postponed</t>
         </is>
       </c>
       <c r="D355" s="4" t="n">
-        <v>10.10989354</v>
-      </c>
-      <c r="E355" s="3" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E355" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F355" s="4" t="n">
-        <v>15.30647778</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356">
@@ -9294,15 +9294,15 @@
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>J-1.a Pending JESA DMR / attachment creation</t>
+          <t>C-4.a Pending client PM approval</t>
         </is>
       </c>
       <c r="D356" s="4" t="n">
-        <v>19.82471001050001</v>
+        <v>10.10989354</v>
       </c>
       <c r="E356" s="3" t="n"/>
       <c r="F356" s="4" t="n">
-        <v>12.0219518505</v>
+        <v>15.30647778</v>
       </c>
     </row>
     <row r="357">
@@ -9318,15 +9318,15 @@
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
+          <t>J-1.a Pending JESA DMR / attachment creation</t>
         </is>
       </c>
       <c r="D357" s="4" t="n">
-        <v>9.438410930000002</v>
+        <v>19.82471001050001</v>
       </c>
       <c r="E357" s="3" t="n"/>
       <c r="F357" s="4" t="n">
-        <v>9.034256850000002</v>
+        <v>12.0219518505</v>
       </c>
     </row>
     <row r="358">
@@ -9342,15 +9342,15 @@
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>C-1.c Pending client PO</t>
+          <t>C-5.a Signed by client PM, pending OCP SS approval</t>
         </is>
       </c>
       <c r="D358" s="4" t="n">
-        <v>4.072588319999999</v>
+        <v>9.438410930000002</v>
       </c>
       <c r="E358" s="3" t="n"/>
       <c r="F358" s="4" t="n">
-        <v>3.55175032</v>
+        <v>9.034256850000002</v>
       </c>
     </row>
     <row r="359">
@@ -9366,15 +9366,15 @@
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>J-4.a Ongoing invoicing</t>
+          <t>C-1.c Pending client PO</t>
         </is>
       </c>
       <c r="D359" s="4" t="n">
-        <v>0.412</v>
+        <v>4.072588319999999</v>
       </c>
       <c r="E359" s="3" t="n"/>
       <c r="F359" s="4" t="n">
-        <v>1.495799</v>
+        <v>3.55175032</v>
       </c>
     </row>
     <row r="360">
@@ -9390,15 +9390,15 @@
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>J-7.a Under investigation</t>
+          <t>J-4.a Ongoing invoicing</t>
         </is>
       </c>
       <c r="D360" s="4" t="n">
-        <v>0.178857745</v>
+        <v>0.412</v>
       </c>
       <c r="E360" s="3" t="n"/>
       <c r="F360" s="4" t="n">
-        <v>0.178857745</v>
+        <v>1.495799</v>
       </c>
     </row>
     <row r="361">
@@ -9414,15 +9414,15 @@
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>C-6.a Pending SS OCP rejection</t>
+          <t>J-7.a Under investigation</t>
         </is>
       </c>
       <c r="D361" s="4" t="n">
-        <v>1.495799</v>
+        <v>0.178857745</v>
       </c>
       <c r="E361" s="3" t="n"/>
       <c r="F361" s="4" t="n">
-        <v>0</v>
+        <v>0.178857745</v>
       </c>
     </row>
     <row r="362">
@@ -9433,20 +9433,20 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>C-6.a Pending SS OCP rejection</t>
         </is>
       </c>
       <c r="D362" s="4" t="n">
-        <v>7.620723</v>
+        <v>1.495799</v>
       </c>
       <c r="E362" s="3" t="n"/>
       <c r="F362" s="4" t="n">
-        <v>8.241983000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363">
@@ -9462,15 +9462,15 @@
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D363" s="4" t="n">
-        <v>19.8199807618</v>
+        <v>7.620723</v>
       </c>
       <c r="E363" s="3" t="n"/>
       <c r="F363" s="4" t="n">
-        <v>20.0097067618</v>
+        <v>8.241983000000001</v>
       </c>
     </row>
     <row r="364">
@@ -9486,15 +9486,15 @@
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D364" s="4" t="n">
-        <v>0</v>
+        <v>19.8199807618</v>
       </c>
       <c r="E364" s="3" t="n"/>
       <c r="F364" s="4" t="n">
-        <v>0</v>
+        <v>20.0097067618</v>
       </c>
     </row>
     <row r="365">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D365" s="4" t="n">
@@ -9529,20 +9529,20 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D366" s="4" t="n">
-        <v>5.702727</v>
+        <v>0</v>
       </c>
       <c r="E366" s="3" t="n"/>
       <c r="F366" s="4" t="n">
-        <v>5.702727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="367">
@@ -9558,15 +9558,15 @@
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D367" s="4" t="n">
-        <v>0.266</v>
+        <v>5.702727</v>
       </c>
       <c r="E367" s="3" t="n"/>
       <c r="F367" s="4" t="n">
-        <v>0.266</v>
+        <v>5.702727</v>
       </c>
     </row>
     <row r="368">
@@ -9582,15 +9582,15 @@
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D368" s="4" t="n">
-        <v>0</v>
+        <v>0.266</v>
       </c>
       <c r="E368" s="3" t="n"/>
       <c r="F368" s="4" t="n">
-        <v>0</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="369">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D369" s="4" t="n">
@@ -9630,15 +9630,15 @@
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D370" s="4" t="n">
-        <v>5.599305</v>
+        <v>0</v>
       </c>
       <c r="E370" s="3" t="n"/>
       <c r="F370" s="4" t="n">
-        <v>3.010328</v>
+        <v>0</v>
       </c>
     </row>
     <row r="371">
@@ -9654,15 +9654,15 @@
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D371" s="4" t="n">
-        <v>0</v>
+        <v>5.599305</v>
       </c>
       <c r="E371" s="3" t="n"/>
       <c r="F371" s="4" t="n">
-        <v>0</v>
+        <v>3.010328</v>
       </c>
     </row>
     <row r="372">
@@ -9678,7 +9678,7 @@
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D372" s="4" t="n">
@@ -9702,15 +9702,15 @@
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D373" s="4" t="n">
-        <v>15.8726717618</v>
+        <v>0</v>
       </c>
       <c r="E373" s="3" t="n"/>
       <c r="F373" s="4" t="n">
-        <v>19.2726347618</v>
+        <v>0</v>
       </c>
     </row>
     <row r="374">
@@ -9721,20 +9721,20 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D374" s="4" t="n">
-        <v>7.449941010000002</v>
+        <v>15.8726717618</v>
       </c>
       <c r="E374" s="3" t="n"/>
       <c r="F374" s="4" t="n">
-        <v>7.500495880000001</v>
+        <v>19.2726347618</v>
       </c>
     </row>
     <row r="375">
@@ -9745,7 +9745,7 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
@@ -9754,11 +9754,11 @@
         </is>
       </c>
       <c r="D375" s="4" t="n">
-        <v>1.966475</v>
+        <v>7.449941010000002</v>
       </c>
       <c r="E375" s="3" t="n"/>
       <c r="F375" s="4" t="n">
-        <v>6.410291</v>
+        <v>7.500495880000001</v>
       </c>
     </row>
     <row r="376">
@@ -9769,20 +9769,20 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D376" s="4" t="n">
-        <v>3.019860209999999</v>
+        <v>1.966475</v>
       </c>
       <c r="E376" s="3" t="n"/>
       <c r="F376" s="4" t="n">
-        <v>2.776067639999999</v>
+        <v>6.410291</v>
       </c>
     </row>
     <row r="377">
@@ -9793,7 +9793,7 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
@@ -9802,11 +9802,11 @@
         </is>
       </c>
       <c r="D377" s="4" t="n">
-        <v>3.31</v>
+        <v>3.019860209999999</v>
       </c>
       <c r="E377" s="3" t="n"/>
       <c r="F377" s="4" t="n">
-        <v>0</v>
+        <v>2.776067639999999</v>
       </c>
     </row>
     <row r="378">
@@ -9817,20 +9817,20 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D378" s="4" t="n">
-        <v>5.90244817</v>
+        <v>3.31</v>
       </c>
       <c r="E378" s="3" t="n"/>
       <c r="F378" s="4" t="n">
-        <v>5.09577917</v>
+        <v>0</v>
       </c>
     </row>
     <row r="379">
@@ -9841,7 +9841,7 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
@@ -9850,11 +9850,11 @@
         </is>
       </c>
       <c r="D379" s="4" t="n">
-        <v>3.330940422</v>
+        <v>5.90244817</v>
       </c>
       <c r="E379" s="3" t="n"/>
       <c r="F379" s="4" t="n">
-        <v>3.330940422</v>
+        <v>5.09577917</v>
       </c>
     </row>
     <row r="380">
@@ -9865,20 +9865,20 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D380" s="4" t="n">
-        <v>1.97228386</v>
+        <v>3.330940422</v>
       </c>
       <c r="E380" s="3" t="n"/>
       <c r="F380" s="4" t="n">
-        <v>1.97228386</v>
+        <v>3.330940422</v>
       </c>
     </row>
     <row r="381">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
@@ -9898,11 +9898,11 @@
         </is>
       </c>
       <c r="D381" s="4" t="n">
-        <v>10.3206683398</v>
+        <v>1.97228386</v>
       </c>
       <c r="E381" s="3" t="n"/>
       <c r="F381" s="4" t="n">
-        <v>10.3206683398</v>
+        <v>1.97228386</v>
       </c>
     </row>
     <row r="382">
@@ -9913,20 +9913,20 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D382" s="4" t="n">
-        <v>27.1877262955</v>
+        <v>10.3206683398</v>
       </c>
       <c r="E382" s="3" t="n"/>
       <c r="F382" s="4" t="n">
-        <v>24.2444669955</v>
+        <v>10.3206683398</v>
       </c>
     </row>
     <row r="383">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
@@ -9946,11 +9946,11 @@
         </is>
       </c>
       <c r="D383" s="4" t="n">
-        <v>8.51262</v>
+        <v>27.1877262955</v>
       </c>
       <c r="E383" s="3" t="n"/>
       <c r="F383" s="4" t="n">
-        <v>8.18979</v>
+        <v>24.2444669955</v>
       </c>
     </row>
     <row r="384">
@@ -9961,20 +9961,20 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D384" s="4" t="n">
-        <v>0</v>
+        <v>8.51262</v>
       </c>
       <c r="E384" s="3" t="n"/>
       <c r="F384" s="4" t="n">
-        <v>0</v>
+        <v>8.18979</v>
       </c>
     </row>
     <row r="385">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
@@ -10004,25 +10004,23 @@
     <row r="386">
       <c r="A386" s="3" t="inlineStr">
         <is>
-          <t>Building &amp; Capabilities</t>
+          <t>Advisory</t>
         </is>
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D386" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E386" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="E386" s="3" t="n"/>
       <c r="F386" s="4" t="n">
         <v>0</v>
       </c>
@@ -10040,17 +10038,17 @@
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Under JESA</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="D387" s="4" t="n">
-        <v>2.04183504</v>
+        <v>0</v>
       </c>
       <c r="E387" s="4" t="n">
-        <v>2.04183504</v>
+        <v>0</v>
       </c>
       <c r="F387" s="4" t="n">
-        <v>2.04183504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="388">
@@ -10066,17 +10064,17 @@
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Under OCP</t>
+          <t>Under JESA</t>
         </is>
       </c>
       <c r="D388" s="4" t="n">
-        <v>3.94193829</v>
+        <v>2.04183504</v>
       </c>
       <c r="E388" s="4" t="n">
-        <v>3.941938290000001</v>
+        <v>2.04183504</v>
       </c>
       <c r="F388" s="4" t="n">
-        <v>3.94193829</v>
+        <v>2.04183504</v>
       </c>
     </row>
     <row r="389">
@@ -10092,17 +10090,17 @@
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>SS postponed</t>
+          <t>Under OCP</t>
         </is>
       </c>
       <c r="D389" s="4" t="n">
-        <v>0</v>
+        <v>3.94193829</v>
       </c>
       <c r="E389" s="4" t="n">
-        <v>0</v>
+        <v>3.941938290000001</v>
       </c>
       <c r="F389" s="4" t="n">
-        <v>0</v>
+        <v>3.94193829</v>
       </c>
     </row>
     <row r="390">
@@ -10113,20 +10111,22 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>unbilled_status</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>C-4.a Pending client PM approval</t>
+          <t>SS postponed</t>
         </is>
       </c>
       <c r="D390" s="4" t="n">
-        <v>3.94193829</v>
-      </c>
-      <c r="E390" s="3" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E390" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F390" s="4" t="n">
-        <v>3.94193829</v>
+        <v>0</v>
       </c>
     </row>
     <row r="391">
@@ -10142,15 +10142,15 @@
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>J-1.b Pending attachments JESA PA</t>
+          <t>C-4.a Pending client PM approval</t>
         </is>
       </c>
       <c r="D391" s="4" t="n">
-        <v>1.42969378</v>
+        <v>3.94193829</v>
       </c>
       <c r="E391" s="3" t="n"/>
       <c r="F391" s="4" t="n">
-        <v>1.42969378</v>
+        <v>3.94193829</v>
       </c>
     </row>
     <row r="392">
@@ -10166,15 +10166,15 @@
       </c>
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>J-2.a Pending JESA PM approval</t>
+          <t>J-1.b Pending attachments JESA PA</t>
         </is>
       </c>
       <c r="D392" s="4" t="n">
-        <v>0.61214126</v>
+        <v>1.42969378</v>
       </c>
       <c r="E392" s="3" t="n"/>
       <c r="F392" s="4" t="n">
-        <v>0.61214126</v>
+        <v>1.42969378</v>
       </c>
     </row>
     <row r="393">
@@ -10185,20 +10185,20 @@
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>unpaid_group</t>
+          <t>unbilled_status</t>
         </is>
       </c>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
       <c r="D393" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0.61214126</v>
       </c>
       <c r="E393" s="3" t="n"/>
       <c r="F393" s="4" t="n">
-        <v>0</v>
+        <v>0.61214126</v>
       </c>
     </row>
     <row r="394">
@@ -10214,15 +10214,15 @@
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>Past due</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="D394" s="4" t="n">
-        <v>1.08369285</v>
+        <v>0.3396483899999996</v>
       </c>
       <c r="E394" s="3" t="n"/>
       <c r="F394" s="4" t="n">
-        <v>1.42334124</v>
+        <v>0</v>
       </c>
     </row>
     <row r="395">
@@ -10238,15 +10238,15 @@
       </c>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Past due</t>
         </is>
       </c>
       <c r="D395" s="4" t="n">
-        <v>0</v>
+        <v>1.08369285</v>
       </c>
       <c r="E395" s="3" t="n"/>
       <c r="F395" s="4" t="n">
-        <v>0</v>
+        <v>1.42334124</v>
       </c>
     </row>
     <row r="396">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D396" s="4" t="n">
@@ -10281,12 +10281,12 @@
       </c>
       <c r="B397" s="3" t="inlineStr">
         <is>
-          <t>unpaid_phase</t>
+          <t>unpaid_group</t>
         </is>
       </c>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D397" s="4" t="n">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="D398" s="4" t="n">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>OCP subs</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="D399" s="4" t="n">
@@ -10358,15 +10358,15 @@
       </c>
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>Ordonnancement</t>
+          <t>OCP subs</t>
         </is>
       </c>
       <c r="D400" s="4" t="n">
-        <v>1.08369285</v>
+        <v>0</v>
       </c>
       <c r="E400" s="3" t="n"/>
       <c r="F400" s="4" t="n">
-        <v>1.08369285</v>
+        <v>0</v>
       </c>
     </row>
     <row r="401">
@@ -10382,15 +10382,15 @@
       </c>
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>Missing reception</t>
+          <t>Ordonnancement</t>
         </is>
       </c>
       <c r="D401" s="4" t="n">
-        <v>0</v>
+        <v>1.08369285</v>
       </c>
       <c r="E401" s="3" t="n"/>
       <c r="F401" s="4" t="n">
-        <v>0</v>
+        <v>1.08369285</v>
       </c>
     </row>
     <row r="402">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>Non-OCP / OCP sub (hors)</t>
+          <t>Missing reception</t>
         </is>
       </c>
       <c r="D402" s="4" t="n">
@@ -10430,7 +10430,7 @@
       </c>
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>Being processed</t>
+          <t>Non-OCP / OCP sub (hors)</t>
         </is>
       </c>
       <c r="D403" s="4" t="n">
@@ -10454,15 +10454,15 @@
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Being processed</t>
         </is>
       </c>
       <c r="D404" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0</v>
       </c>
       <c r="E404" s="3" t="n"/>
       <c r="F404" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0</v>
       </c>
     </row>
     <row r="405">
@@ -10473,20 +10473,20 @@
       </c>
       <c r="B405" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>unpaid_phase</t>
         </is>
       </c>
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D405" s="4" t="n">
-        <v>0.4907168099999997</v>
+        <v>0.3396483899999996</v>
       </c>
       <c r="E405" s="3" t="n"/>
       <c r="F405" s="4" t="n">
-        <v>0.4907168099999997</v>
+        <v>0.3396483899999996</v>
       </c>
     </row>
     <row r="406">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B406" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C406" s="3" t="inlineStr">
@@ -10506,11 +10506,11 @@
         </is>
       </c>
       <c r="D406" s="4" t="n">
-        <v>0</v>
+        <v>0.4907168099999997</v>
       </c>
       <c r="E406" s="3" t="n"/>
       <c r="F406" s="4" t="n">
-        <v>0</v>
+        <v>0.4907168099999997</v>
       </c>
     </row>
     <row r="407">
@@ -10521,20 +10521,20 @@
       </c>
       <c r="B407" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C407" s="3" t="inlineStr">
         <is>
-          <t>31–60 days</t>
+          <t>&lt; 30 days</t>
         </is>
       </c>
       <c r="D407" s="4" t="n">
-        <v>0.22973683</v>
+        <v>0</v>
       </c>
       <c r="E407" s="3" t="n"/>
       <c r="F407" s="4" t="n">
-        <v>0.22973683</v>
+        <v>0</v>
       </c>
     </row>
     <row r="408">
@@ -10545,7 +10545,7 @@
       </c>
       <c r="B408" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C408" s="3" t="inlineStr">
@@ -10554,11 +10554,11 @@
         </is>
       </c>
       <c r="D408" s="4" t="n">
-        <v>0.7691738100000001</v>
+        <v>0.22973683</v>
       </c>
       <c r="E408" s="3" t="n"/>
       <c r="F408" s="4" t="n">
-        <v>0.7691738100000001</v>
+        <v>0.22973683</v>
       </c>
     </row>
     <row r="409">
@@ -10569,20 +10569,20 @@
       </c>
       <c r="B409" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C409" s="3" t="inlineStr">
         <is>
-          <t>61–90 days</t>
+          <t>31–60 days</t>
         </is>
       </c>
       <c r="D409" s="4" t="n">
-        <v>0.6202166199999994</v>
+        <v>0.7691738100000001</v>
       </c>
       <c r="E409" s="3" t="n"/>
       <c r="F409" s="4" t="n">
-        <v>0.6202166199999994</v>
+        <v>0.7691738100000001</v>
       </c>
     </row>
     <row r="410">
@@ -10593,7 +10593,7 @@
       </c>
       <c r="B410" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C410" s="3" t="inlineStr">
@@ -10602,11 +10602,11 @@
         </is>
       </c>
       <c r="D410" s="4" t="n">
-        <v>0.31451904</v>
+        <v>0.6202166199999994</v>
       </c>
       <c r="E410" s="3" t="n"/>
       <c r="F410" s="4" t="n">
-        <v>0.31451904</v>
+        <v>0.6202166199999994</v>
       </c>
     </row>
     <row r="411">
@@ -10617,20 +10617,20 @@
       </c>
       <c r="B411" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>91–120 days</t>
+          <t>61–90 days</t>
         </is>
       </c>
       <c r="D411" s="4" t="n">
-        <v>0.8676346699999999</v>
+        <v>0.31451904</v>
       </c>
       <c r="E411" s="3" t="n"/>
       <c r="F411" s="4" t="n">
-        <v>0.8676346699999999</v>
+        <v>0.31451904</v>
       </c>
     </row>
     <row r="412">
@@ -10641,7 +10641,7 @@
       </c>
       <c r="B412" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C412" s="3" t="inlineStr">
@@ -10650,11 +10650,11 @@
         </is>
       </c>
       <c r="D412" s="4" t="n">
-        <v>0</v>
+        <v>0.8676346699999999</v>
       </c>
       <c r="E412" s="3" t="n"/>
       <c r="F412" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0.8676346699999999</v>
       </c>
     </row>
     <row r="413">
@@ -10665,20 +10665,20 @@
       </c>
       <c r="B413" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>&gt; 120 days</t>
+          <t>91–120 days</t>
         </is>
       </c>
       <c r="D413" s="4" t="n">
-        <v>3.775468400000001</v>
+        <v>0</v>
       </c>
       <c r="E413" s="3" t="n"/>
       <c r="F413" s="4" t="n">
-        <v>3.775468400000001</v>
+        <v>0.3396483899999996</v>
       </c>
     </row>
     <row r="414">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B414" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C414" s="3" t="inlineStr">
@@ -10698,11 +10698,11 @@
         </is>
       </c>
       <c r="D414" s="4" t="n">
-        <v>0</v>
+        <v>3.775468400000001</v>
       </c>
       <c r="E414" s="3" t="n"/>
       <c r="F414" s="4" t="n">
-        <v>0</v>
+        <v>3.775468400000001</v>
       </c>
     </row>
     <row r="415">
@@ -10713,12 +10713,12 @@
       </c>
       <c r="B415" s="3" t="inlineStr">
         <is>
-          <t>aging_unbilled</t>
+          <t>aging_unpaid</t>
         </is>
       </c>
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>&gt; 120 days</t>
         </is>
       </c>
       <c r="D415" s="4" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B416" s="3" t="inlineStr">
         <is>
-          <t>aging_unpaid</t>
+          <t>aging_unbilled</t>
         </is>
       </c>
       <c r="C416" s="3" t="inlineStr">
@@ -10746,10 +10746,34 @@
         </is>
       </c>
       <c r="D416" s="4" t="n">
-        <v>0.3396483899999996</v>
+        <v>0</v>
       </c>
       <c r="E416" s="3" t="n"/>
       <c r="F416" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B417" s="3" t="inlineStr">
+        <is>
+          <t>aging_unpaid</t>
+        </is>
+      </c>
+      <c r="C417" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D417" s="4" t="n">
+        <v>0.3396483899999996</v>
+      </c>
+      <c r="E417" s="3" t="n"/>
+      <c r="F417" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -19523,12 +19547,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Total AR 12,395 MMAD: −294 vs 14 Oct, −456 vs 07 Oct</t>
+          <t>Total AR 12,397 MMAD: −292 vs 14 Oct, −456 vs 07 Oct</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Unbilled 9,477 (−37 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unbilled under JESA responsibility 720 MMAD (PSR 228 / Procurement 492); non-OCP receivables 252 MMAD.</t>
+          <t>Unbilled 9,479 (−35 WoW), unpaid 2,370 (−257 WoW), advance 548 (0 WoW). Unbilled under JESA responsibility 720 MMAD (PSR 228 / Procurement 492); non-OCP receivables 252 MMAD.</t>
         </is>
       </c>
     </row>
@@ -19538,7 +19562,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Unrecognized revenue 7,128 MMAD (−40 WoW, −424 vs 07 Oct); gross exposure 19,523 MMAD (−334 WoW)</t>
+          <t>Unrecognized revenue 7,128 MMAD (−40 WoW, −424 vs 07 Oct); gross exposure 19,525 MMAD (−332 WoW)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -22796,13 +22820,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>9681.98338223431</v>
+        <v>9683.62880464431</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>9513.792499159648</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>9477.458001200219</v>
+        <v>9479.103423610219</v>
       </c>
     </row>
     <row r="5">
@@ -22828,13 +22852,13 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>12851.26285520714</v>
+        <v>12852.90827761714</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>12688.97665804529</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>12395.06650422525</v>
+        <v>12396.71192663525</v>
       </c>
     </row>
     <row r="7">
@@ -22860,13 +22884,13 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>20403.26285520714</v>
+        <v>20404.90827761714</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>19856.97665804529</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>19523.39533804451</v>
+        <v>19525.04076045451</v>
       </c>
     </row>
     <row r="9">
@@ -29905,7 +29929,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8107.063599238703</v>
+        <v>8108.709021648703</v>
       </c>
     </row>
     <row r="5">
@@ -29925,7 +29949,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>6220.412640508043</v>
+        <v>6222.058062918043</v>
       </c>
     </row>
     <row r="7">
@@ -29955,7 +29979,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>12143.5245726081</v>
+        <v>12145.1699950181</v>
       </c>
     </row>
     <row r="10">
@@ -30560,13 +30584,13 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>145.8125589700002</v>
+        <v>147.4579813800002</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>145.5530990800001</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>145.0767065300002</v>
+        <v>146.7221289400002</v>
       </c>
     </row>
     <row r="29">
@@ -30602,13 +30626,13 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>485.4054907504762</v>
+        <v>487.0509131604763</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>486.3849952404764</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>487.0737428704763</v>
+        <v>488.7191652804763</v>
       </c>
     </row>
     <row r="31">
@@ -31686,13 +31710,13 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>108.7051785900001</v>
+        <v>110.3506010000001</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>108.70517859</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>108.39274161</v>
+        <v>110.03816402</v>
       </c>
     </row>
     <row r="30">
@@ -31979,7 +32003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -32472,17 +32496,17 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>C-2.a Waiting OCP VAT exemption</t>
+          <t>C-3.a Pending DP payment / clearing</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1.50242933</v>
+        <v>1.64542241</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>1.50242933</v>
+        <v>0</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>1.50242933</v>
+        <v>1.64542241</v>
       </c>
     </row>
     <row r="25">
@@ -32493,17 +32517,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>C-1.e Waiting mirror POs for PDR</t>
+          <t>C-2.a Waiting OCP VAT exemption</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0.10387899</v>
+        <v>1.50242933</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0</v>
+        <v>1.50242933</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.10387899</v>
+        <v>1.50242933</v>
       </c>
     </row>
     <row r="26">
@@ -32514,37 +32538,58 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PENDING OCP </t>
+          <t>C-1.e Waiting mirror POs for PDR</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>0</v>
+        <v>0.10387899</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0</v>
+        <v>0.10387899</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t>OCP</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PENDING OCP </t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>JESA</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>J-2.a Pending JESA PM approval</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C28" s="4" t="n">
         <v>-46.80343063892482</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D28" s="4" t="n">
         <v>-62.59554572227994</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E28" s="4" t="n">
         <v>-95.28123365227995</v>
       </c>
     </row>
@@ -32877,13 +32922,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>8275.464593566185</v>
+        <v>8277.110015976186</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>8120.680624622309</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>8017.265084642301</v>
+        <v>8018.910507052301</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Deck feedback round: variance pills, DSO/paid on summary, BU heat table, non-OCP paid, PSR slide
- Title: info line removed, WoW variance shown as bold coloured MDH pills
- AR executive summary: smaller OCP share callout plus DSO, paid and deposited cards
- AR movement: BU heat table replaces the narrative; component deltas as green/red bars
- Paid-in-month column on AR by BU, non-OCP paid on the non-OCP and collections slides
- New PSR (labor) collections slide after cash by BU (by BU, provisions, available)
- BU zoom pages carry paid figures; engine splits collections OCP / non-OCP;
  extractor adds CASH_PSR_BU tab and provision lines

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -29,15 +29,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_PSR_BU" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19642,7 +19643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19653,12 +19654,16 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Payments received by BU (amount invoiced, by payment date): current month to 2026-10-20 vs to 2026-10-14, prior full month, YTD; deposited_month = invoices received (reception date) in the current month, HT.</t>
+          <t>Payments received by BU (amount invoiced, by payment date): current month to 2026-10-20 vs to 2026-10-14, prior full month, YTD; deposited_month = invoices received (reception date) in the current month, HT; nonocp_* = same measures for non-OCP clients (Client 1).</t>
         </is>
       </c>
     </row>
@@ -19703,6 +19708,26 @@
           <t>deposited_month</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>nonocp_month_prev_week</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>nonocp_month_current</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>nonocp_prior_month</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>nonocp_ytd</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -19731,6 +19756,18 @@
       <c r="H3" s="4" t="n">
         <v>0.16916875</v>
       </c>
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.24567691</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>3.51085755</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -19759,6 +19796,18 @@
       <c r="H4" s="4" t="n">
         <v>70.37159896999995</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -19787,6 +19836,18 @@
       <c r="H5" s="4" t="n">
         <v>27.70975094</v>
       </c>
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>2.64395687</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>2.64395687</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -19815,6 +19876,18 @@
       <c r="H6" s="4" t="n">
         <v>1.649866900000006</v>
       </c>
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -19843,6 +19916,18 @@
       <c r="H7" s="4" t="n">
         <v>5.242102080442559</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>3.1264161761136</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>3.1264161761136</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>2.2342086</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>25.3939867546076</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -19871,6 +19956,18 @@
       <c r="H8" s="4" t="n">
         <v>15.854857709692</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>7.603861025670001</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>7.603861025670001</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>22.03586198064</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>117.1772017279</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -19899,6 +19996,18 @@
       <c r="H9" s="4" t="n">
         <v>4.05677018907</v>
       </c>
+      <c r="I9" s="4" t="n">
+        <v>2.99184</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>7.713264910000001</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>20.95615629</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>63.649580586592</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -19927,6 +20036,18 @@
       <c r="H10" s="4" t="n">
         <v>10.27366639</v>
       </c>
+      <c r="I10" s="4" t="n">
+        <v>0.634778352</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.846371136</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>8.107821387</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -19955,6 +20076,18 @@
       <c r="H11" s="4" t="n">
         <v>8.699596000000001</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>2.606939784000001</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>12.6583916694</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -19981,6 +20114,18 @@
         <v>11</v>
       </c>
       <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20194,7 +20339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -20550,12 +20695,404 @@
         <v>72.82105018999999</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>PSR provision – AM ring-fence</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>-64.6905184</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>-39.86521105000001</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>-39.98830501</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>-54.84980808999999</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>-199.39384255</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>PSR provision – W&amp;E reserve</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>-33.33333333333333</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>-33.33333333333333</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>-33.33333333333333</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Overhead payments (FYI, not deducted)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>-17.58143615</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>-3.01361609</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>-21.21210081965499</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>-2.06410341</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>-2.65077389</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>-46.52203035965499</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PSR (labor) collections by BU per OCP payment report (EXEC Summary section 3), MMAD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>jul</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>aug</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>sep</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>oct_actual</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>oct_ongoing</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>cumulative</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>64.6905184</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>39.86521105000001</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>39.98830501</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>54.84980808999999</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>199.39384255</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>2.358803</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>12.149944</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>10.772904</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>25.281651</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0.46304705</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1.79696815</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2.74066266</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>5.00067786</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0.67352388</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>6.015997110000001</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>2.86983472</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.44352734</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>10.00288305</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>4.22674162</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>6.417104190000001</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>7.834129519999999</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>18.47797533</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>7.55665327</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0.9863724</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.50618315</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>9.04920882</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>3.41382482</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>3.41382482</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>15.47090669</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>85.70278394999998</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.42113867</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>101.59482931</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20980,7 +21517,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21297,7 +21834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21556,7 +22093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21945,7 +22482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22153,7 +22690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22609,143 +23146,6 @@
       </c>
       <c r="D25" s="3" t="n">
         <v>64</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Supplier invoice file: open payables by supplier tier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>tier</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>1 - National</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>837.2819903599992</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2 - National</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>480.1798277400004</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>International</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>460.645999433202</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>1 - International</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>159.1098221761841</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>2 - International</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>71.59981245506602</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>3 - National</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>46.01373270000001</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Not on OCP Tier</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>45.52547409999993</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Office/Publique</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>31.80906488</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>OCP et Filiale</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>8.973442450000002</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>3 - International</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>2.4342852509</v>
       </c>
     </row>
   </sheetData>
@@ -22984,6 +23384,143 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Supplier invoice file: open payables by supplier tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1 - National</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>837.2819903599992</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2 - National</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>480.1798277400004</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>460.645999433202</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>1 - International</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>159.1098221761841</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2 - International</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>71.59981245506602</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>3 - National</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>46.01373270000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Not on OCP Tier</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>45.52547409999993</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Office/Publique</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>31.80906488</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>OCP et Filiale</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>8.973442450000002</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>3 - International</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>2.4342852509</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -23246,7 +23783,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
DSO computed from the AR extract and the DSO calculation workbook; DSO trend backup slide
- extract_inputs: --dso-calc reads '12 Months Trailing' (revenue per BU) and
  'Trend'; DSO = total AR / 12m revenue x 365, reproduces the workbook table
  (NOTE printed when the table carries an override); DSO and DSO_TREND tabs
- build_deck: line-chart helper and 'DSO - trend by business unit' backup slide
- run_week.sh picks up *DSO*.xlsx and keeps the latest in inputs/dso_calc/
- README and playbook updated; the BU meeting PDF is no longer needed for DSO

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
+++ b/weekly-ar-cash-deck/inputs/history/weekly_inputs_2026-10-21.xlsx
@@ -26,19 +26,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JESA_UNBILLED_BU" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JESA_UNBILLED_STATUS" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DSO" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_PSR_BU" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DSO_TREND" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_PSR_BU" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19326,18 +19327,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DSO excluding advances (days), from the BU meeting Power BI report. Update monthly; 'JESA Group' row = group DSO.</t>
+          <t>DSO (days) = total AR of the BU / 12-month trailing revenue x 365 (DSO calc workbook); 'JESA Group' row = group DSO; prior month from the Trend sheet.</t>
         </is>
       </c>
     </row>
@@ -19357,29 +19360,53 @@
           <t>dso_prior_month</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>total_ar</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>revenue_12m</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>JESA Group</t>
+          <t>Global Mining</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>285</v>
-      </c>
-      <c r="C3" s="3" t="n"/>
+        <v>252</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>218</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>551.2691067924734</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>799.4392640999999</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Water &amp; Environment</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>331</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>318</v>
+        <v>134</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>893.3956311382896</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>2442.073012560003</v>
       </c>
     </row>
     <row r="5">
@@ -19391,112 +19418,164 @@
       <c r="B5" s="3" t="n">
         <v>376</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>331</v>
+      <c r="C5" s="4" t="n">
+        <v>336</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>3218.868689557612</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>3122.407874849999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>SP2M Ad Hoc Program</t>
+          <t>Water &amp; Environment</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>294</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>268</v>
+        <v>331</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>318</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>3324.59586137112</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>3670.35279131</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>JESA Technologies</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>134</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>135</v>
+        <v>106</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>106.6324758991395</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>368.0652618399999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Global Mining</t>
+          <t>Energy Operations</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>252</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>216</v>
+        <v>190</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>499.8689366197487</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>960.3098550598286</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Building &amp; Infrastructure</t>
+          <t>Advisory</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>462</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>415</v>
+        <v>192</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>203</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>69.84078330730001</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>132.6002191199999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Energy Operations</t>
+          <t>Building &amp; Infrastructure</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>190</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>174</v>
+        <v>462</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>418</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>488.7191652804763</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>386.0175523454156</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Advisory</t>
+          <t>SP2M Ad Hoc Program</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>192</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>203</v>
+        <v>294</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>266</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>3236.114162099108</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>4012.848443020002</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>JESA Technologies</t>
+          <t>Building &amp; Capabilities</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>95</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>107</v>
+        <v>323</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>317</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>7.407114570000001</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>8.38029777</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Building &amp; Capabilities</t>
+          <t>JESA Group</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>323</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>317</v>
+        <v>285</v>
+      </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="4" t="n">
+        <v>12396.71192663527</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>15902.49457197525</v>
       </c>
     </row>
   </sheetData>
@@ -19638,6 +19717,529 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DSO history by BU (days) from the DSO calc workbook 'Trend' sheet; 12-month revenue window Oct-25 to Sep-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Nov-25</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Dec-25</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>188</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>189</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>185</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>170</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>170</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>185</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>197</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>213</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>218</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>144</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>132</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>196</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>192</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>254</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>251</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>252</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>295</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>284</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>310</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>326</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>321</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>336</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>134</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>189</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>144</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>213</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>262</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>260</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>291</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>286</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>279</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>318</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>102</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>159</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>159</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>182</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>187</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>136</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>182</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>181</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>198</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>223</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>203</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>232</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>246</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>268</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>293</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>295</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>322</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>348</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>385</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>418</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>138</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>139</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>134</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>134</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>224</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>240</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>259</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>272</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>266</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="4" t="n">
+        <v>294</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>294</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>311</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>315</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>317</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>323</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20134,7 +20736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20333,7 +20935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20775,7 +21377,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21092,7 +21694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21517,7 +22119,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21834,7 +22436,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22093,7 +22695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22482,7 +23084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22683,469 +23285,6 @@
       </c>
       <c r="C13" s="4" t="n">
         <v>431.3736114969632</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Supplier invoice file: open payables by BU and origin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>bu</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>origin</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>lines</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Downpayment</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>9.696841374999996</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>189.6271102799999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>277.1518968970307</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Advisory</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0.16960679</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Building &amp; Infrastructure</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Downpayment</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>2.835</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Building &amp; Infrastructure</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>3.666297630000001</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Building &amp; Infrastructure</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>1.47922066</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Energy Operations</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>49.30623534000001</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Energy Operations</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>29.40226152</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Fertilizers &amp; Chemicals</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Downpayment</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>75.11919636388802</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Fertilizers &amp; Chemicals</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>106.01826818</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Fertilizers &amp; Chemicals</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>68.44753432219999</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Global Mining</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Downpayment</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>6.180616860000001</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Global Mining</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>16.68518353000001</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Global Mining</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>16.230406602655</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>JESA Technologies</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>13.11764809</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>JESA Technologies</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>18.551859047984</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>SP2M Ad Hoc Program</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Downpayment</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>178.5140971678009</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>SP2M Ad Hoc Program</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>341.7290997300001</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>SP2M Ad Hoc Program</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>391.6898560592921</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Water &amp; Environment</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Downpayment</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="n">
-        <v>25.026686727405</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Water &amp; Environment</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Invoices - 4411</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>89.68438290000003</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Water &amp; Environment</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Parked Invoice</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>233.244145472096</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -23384,6 +23523,469 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Supplier invoice file: open payables by BU and origin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>origin</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Downpayment</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>9.696841374999996</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>189.6271102799999</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>277.1518968970307</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.16960679</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Downpayment</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2.835</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>3.666297630000001</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1.47922066</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>49.30623534000001</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>29.40226152</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Downpayment</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>75.11919636388802</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>106.01826818</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>68.44753432219999</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Downpayment</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>6.180616860000001</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>16.68518353000001</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>16.230406602655</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>13.11764809</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>18.551859047984</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Downpayment</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>178.5140971678009</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>341.7290997300001</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>391.6898560592921</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Downpayment</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>25.026686727405</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Invoices - 4411</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>89.68438290000003</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Parked Invoice</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>233.244145472096</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -23515,7 +24117,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23783,7 +24385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>